<commit_message>
Lock trips as tentative, move Cozumel to 6 nights, add final outreach emails, tracker and workbook builder
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/december_pricing.xlsx
+++ b/december-plan/pricing/december_pricing.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="371">
   <si>
     <t xml:space="preserve">Summary — all-in price per person vs ceiling</t>
   </si>
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Prices before any organiser charge, at the airfare midpoint and 2 sharing. Organiser charge under Approach 2 shown separately. Every price rests on advertised or inferred figures; none is a quote.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cozumel, 7 nights (Tue 8 – Tue 15 Dec)</t>
+    <t xml:space="preserve">Cozumel, 6 nights (Tue 8 – Mon 14 Dec)</t>
   </si>
   <si>
     <t xml:space="preserve">Certified</t>
@@ -59,7 +59,7 @@
     <t xml:space="preserve">5-night version, all-in per person</t>
   </si>
   <si>
-    <t xml:space="preserve">Core only (excl. meals, tips, insurance), 7 nights</t>
+    <t xml:space="preserve">Core only (excl. meals, tips, insurance), 6 nights</t>
   </si>
   <si>
     <t xml:space="preserve">Egypt, Marsa Shagra (Sat 2 – Sat 9 Jan)</t>
@@ -179,7 +179,7 @@
     <t xml:space="preserve">Tips and local extras per trip</t>
   </si>
   <si>
-    <t xml:space="preserve">Cozumel, Tue 8 – Tue 15 Dec 2026 (7 nights) and Tue 8 – Sun 13 Dec (5 nights)</t>
+    <t xml:space="preserve">Cozumel, Tue 8 – Mon 14 Dec 2026 (6 nights) and Tue 8 – Sun 13 Dec (5 nights)</t>
   </si>
   <si>
     <t xml:space="preserve">Flight PHL–CZM return, low</t>
@@ -218,12 +218,15 @@
     <t xml:space="preserve">ADVERTISED (snippet); upper of 65–84</t>
   </si>
   <si>
-    <t xml:space="preserve">Nights, 7-night version</t>
+    <t xml:space="preserve">Nights, 6-night version (Tue 8 – Mon 14)</t>
   </si>
   <si>
     <t xml:space="preserve">nights</t>
   </si>
   <si>
+    <t xml:space="preserve">scope change 22 Sep</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nights, 5-night version</t>
   </si>
   <si>
@@ -290,7 +293,7 @@
     <t xml:space="preserve">ADVERTISED (snippet) + INFERRED</t>
   </si>
   <si>
-    <t xml:space="preserve">Certified dive days, 7-night version (Wed–Sun)</t>
+    <t xml:space="preserve">Certified dive days, 6-night version (Wed–Sun)</t>
   </si>
   <si>
     <t xml:space="preserve">days</t>
@@ -302,7 +305,7 @@
     <t xml:space="preserve">Certified dive days, 5-night version (Wed–Sat)</t>
   </si>
   <si>
-    <t xml:space="preserve">Beginner fun-dive days after course, 7-night (Sat–Sun)</t>
+    <t xml:space="preserve">Beginner fun-dive days after course, 6-night (Sat–Sun)</t>
   </si>
   <si>
     <t xml:space="preserve">Beginner fun-dive days after course, 5-night (Sat)</t>
@@ -554,13 +557,13 @@
     <t xml:space="preserve">George is costed as a diving participant. Free places from operators are applied first; any remainder is shown as a disclosed per-head charge.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cozumel — Tue 8 – Tue 15 Dec 2026 (7 nights) and Tue 8 – Sun 13 Dec (5 nights)</t>
+    <t xml:space="preserve">Cozumel — Tue 8 – Mon 14 Dec 2026 (6 nights) and Tue 8 – Sun 13 Dec (5 nights)</t>
   </si>
   <si>
     <t xml:space="preserve">All figures per person, USD. Reads from Inputs. Lodging at Hotel Cozumel &amp; Resort, 2 sharing, breakfast included. Flights at the midpoint of the aggregator band.</t>
   </si>
   <si>
-    <t xml:space="preserve">A. Per-person cost, 7-night version</t>
+    <t xml:space="preserve">A. Per-person cost, 6-night version (no spare day: a norther on Sat/Sun hits the certification dives)</t>
   </si>
   <si>
     <t xml:space="preserve">Item</t>
@@ -629,7 +632,7 @@
     <t xml:space="preserve">B. Per-person cost, 5-night version (Sun 13 return; no norther buffer)</t>
   </si>
   <si>
-    <t xml:space="preserve">C. Organiser place (7-night version), by group size</t>
+    <t xml:space="preserve">C. Organiser place (6-night version), by group size</t>
   </si>
   <si>
     <t xml:space="preserve">20 people</t>
@@ -683,7 +686,7 @@
     <t xml:space="preserve">Unused free places (could offset an instructor or assistant place)</t>
   </si>
   <si>
-    <t xml:space="preserve">D. Sensitivity (7-night version, per person, before organiser charge)</t>
+    <t xml:space="preserve">D. Sensitivity (6-night version, per person, before organiser charge)</t>
   </si>
   <si>
     <t xml:space="preserve">Airfare</t>
@@ -734,7 +737,7 @@
     <t xml:space="preserve">Beginner: only the park fee is MXN-priced; effect under USD 10 per person either way</t>
   </si>
   <si>
-    <t xml:space="preserve">E. Break-even group size (7-night version)</t>
+    <t xml:space="preserve">E. Break-even group size (6-night version)</t>
   </si>
   <si>
     <t xml:space="preserve">Smallest group at which a certified diver stays under the ceiling when George's uncovered cost is spread per head (Approach 2, one free place assumed from 10 paying).</t>
@@ -1539,15 +1542,15 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">Cozumel!B22</f>
-        <v>2334.24434126524</v>
+        <v>2245.24434126524</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Cozumel!C22</f>
-        <v>2429.30528148578</v>
+        <v>2340.30528148578</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">Cozumel!D22</f>
-        <v>3031.24434126524</v>
+        <v>2942.24434126524</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1573,15 +1576,15 @@
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">B8-B7</f>
-        <v>-334.244341265235</v>
+        <v>-245.244341265235</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">C8-C7</f>
-        <v>-129.305281485781</v>
+        <v>-40.3052814857806</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">D8-D7</f>
-        <v>-1031.24434126524</v>
+        <v>-942.244341265235</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1590,15 +1593,15 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Cozumel!B65</f>
-        <v>80.8421052631579</v>
+        <v>76.1578947368421</v>
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Cozumel!C65</f>
-        <v>52.9655172413793</v>
+        <v>49.8965517241379</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">Cozumel!D65</f>
-        <v>39.3846153846154</v>
+        <v>37.1025641025641</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1624,15 +1627,15 @@
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">Cozumel!B23</f>
-        <v>1920.24434126524</v>
+        <v>1866.24434126524</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">Cozumel!C23</f>
-        <v>2015.30528148578</v>
+        <v>1961.30528148578</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">Cozumel!D23</f>
-        <v>2617.24434126524</v>
+        <v>2563.24434126524</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2163,18 +2166,18 @@
         <v>64</v>
       </c>
       <c r="B32" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>37</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B33" s="10" t="n">
         <v>5</v>
@@ -2188,7 +2191,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B34" s="9" t="n">
         <v>400</v>
@@ -2197,12 +2200,12 @@
         <v>41</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B35" s="9" t="n">
         <v>195</v>
@@ -2211,26 +2214,26 @@
         <v>41</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B36" s="11" t="n">
         <v>10500</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B37" s="9" t="n">
         <v>120</v>
@@ -2239,26 +2242,26 @@
         <v>41</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B38" s="11" t="n">
         <v>220</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B39" s="9" t="n">
         <v>25</v>
@@ -2272,7 +2275,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B40" s="9" t="n">
         <v>30</v>
@@ -2281,12 +2284,12 @@
         <v>41</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B41" s="9" t="n">
         <v>530</v>
@@ -2295,12 +2298,12 @@
         <v>41</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B42" s="9" t="n">
         <v>12</v>
@@ -2309,12 +2312,12 @@
         <v>41</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B43" s="9" t="n">
         <v>95</v>
@@ -2328,7 +2331,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B44" s="9" t="n">
         <v>260</v>
@@ -2337,74 +2340,74 @@
         <v>41</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B45" s="10" t="n">
         <v>5</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B46" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B47" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B48" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B49" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>31</v>
@@ -2412,26 +2415,26 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B50" s="10" t="n">
         <v>10</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B53" s="9" t="n">
         <v>700</v>
@@ -2445,7 +2448,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B54" s="9" t="n">
         <v>1300</v>
@@ -2459,7 +2462,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B55" s="9" t="n">
         <v>1300</v>
@@ -2468,12 +2471,12 @@
         <v>41</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B56" s="9" t="n">
         <v>0</v>
@@ -2482,12 +2485,12 @@
         <v>41</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B57" s="10" t="n">
         <v>6</v>
@@ -2496,228 +2499,228 @@
         <v>65</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B58" s="11" t="n">
         <v>78</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B59" s="11" t="n">
         <v>113</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B60" s="11" t="n">
         <v>358</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B61" s="11" t="n">
         <v>94</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B62" s="11" t="n">
         <v>347</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B63" s="11" t="n">
         <v>69</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B64" s="11" t="n">
         <v>15</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B65" s="11" t="n">
         <v>315</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B66" s="11" t="n">
         <v>67</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B67" s="11" t="n">
         <v>59</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B68" s="11" t="n">
         <v>80</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B69" s="11" t="n">
         <v>22</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B70" s="11" t="n">
         <v>17</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B71" s="11" t="n">
         <v>41</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B72" s="11" t="n">
         <v>45</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B73" s="11" t="n">
         <v>7</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>31</v>
@@ -2725,7 +2728,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B74" s="9" t="n">
         <v>15</v>
@@ -2739,41 +2742,41 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B75" s="10" t="n">
         <v>5</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B76" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B77" s="10" t="n">
         <v>11</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>31</v>
@@ -2781,26 +2784,26 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B78" s="10" t="n">
         <v>22</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B81" s="9" t="n">
         <v>400</v>
@@ -2809,12 +2812,12 @@
         <v>41</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B82" s="9" t="n">
         <v>700</v>
@@ -2823,12 +2826,12 @@
         <v>41</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B83" s="10" t="n">
         <v>4</v>
@@ -2842,7 +2845,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B84" s="10" t="n">
         <v>5</v>
@@ -2856,7 +2859,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B85" s="9" t="n">
         <v>75</v>
@@ -2870,7 +2873,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B86" s="9" t="n">
         <v>50</v>
@@ -2884,7 +2887,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B87" s="9" t="n">
         <v>125</v>
@@ -2898,7 +2901,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B88" s="9" t="n">
         <v>140</v>
@@ -2907,54 +2910,54 @@
         <v>41</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B89" s="10" t="n">
         <v>3</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B90" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B91" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B92" s="9" t="n">
         <v>45</v>
@@ -2968,7 +2971,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B93" s="9" t="n">
         <v>70</v>
@@ -2977,26 +2980,26 @@
         <v>41</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B94" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B95" s="9" t="n">
         <v>60</v>
@@ -3010,7 +3013,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B96" s="9" t="n">
         <v>399</v>
@@ -3019,54 +3022,54 @@
         <v>41</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B97" s="8" t="n">
         <v>0.1</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B98" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B99" s="10" t="n">
         <v>3</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B100" s="9" t="n">
         <v>300</v>
@@ -3075,12 +3078,12 @@
         <v>41</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B101" s="9" t="n">
         <v>300</v>
@@ -3089,12 +3092,12 @@
         <v>41</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B102" s="9" t="n">
         <v>240</v>
@@ -3103,12 +3106,12 @@
         <v>41</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B103" s="9" t="n">
         <v>125</v>
@@ -3117,12 +3120,12 @@
         <v>41</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B104" s="9" t="n">
         <v>100</v>
@@ -3136,7 +3139,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B105" s="9" t="n">
         <v>50</v>
@@ -3145,12 +3148,12 @@
         <v>41</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B106" s="9" t="n">
         <v>15</v>
@@ -3164,12 +3167,12 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -3197,22 +3200,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>3</v>
@@ -3226,7 +3229,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$25,Inputs!$B$26)</f>
@@ -3243,7 +3246,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B8" s="4" t="n">
         <f aca="false">2*Inputs!$B$28</f>
@@ -3260,24 +3263,24 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$29</f>
-        <v>378</v>
+        <v>324</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$29</f>
-        <v>378</v>
+        <v>324</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$29</f>
-        <v>378</v>
+        <v>324</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
@@ -3292,7 +3295,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
@@ -3307,7 +3310,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3324,7 +3327,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>0</v>
@@ -3339,7 +3342,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">Inputs!$B$45*Inputs!$B$38/Inputs!$B$7</f>
@@ -3356,7 +3359,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">Inputs!$B$45*Inputs!$B$39</f>
@@ -3373,7 +3376,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">Inputs!$B$40</f>
@@ -3389,7 +3392,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>0</v>
@@ -3404,7 +3407,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>0</v>
@@ -3419,24 +3422,24 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$21</f>
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="C19" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$21</f>
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="D19" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$21</f>
-        <v>245</v>
+        <v>210</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B20" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -3453,7 +3456,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B21" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -3470,41 +3473,41 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">SUM(B7:B21)</f>
-        <v>2334.24434126524</v>
+        <v>2245.24434126524</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">SUM(C7:C21)</f>
-        <v>2429.30528148578</v>
+        <v>2340.30528148578</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">SUM(D7:D21)</f>
-        <v>3031.24434126524</v>
+        <v>2942.24434126524</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B23" s="4" t="n">
         <f aca="false">B22-SUM(B19:B21)</f>
-        <v>1920.24434126524</v>
+        <v>1866.24434126524</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">C22-SUM(C19:C21)</f>
-        <v>2015.30528148578</v>
+        <v>1961.30528148578</v>
       </c>
       <c r="D23" s="4" t="n">
         <f aca="false">D22-SUM(D19:D21)</f>
-        <v>2617.24434126524</v>
+        <v>2563.24434126524</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B24" s="4" t="n">
         <f aca="false">Inputs!$B$15</f>
@@ -3521,24 +3524,24 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B25" s="4" t="n">
         <f aca="false">B24-B22</f>
-        <v>-334.244341265235</v>
+        <v>-245.244341265235</v>
       </c>
       <c r="C25" s="4" t="n">
         <f aca="false">C24-C22</f>
-        <v>-129.305281485781</v>
+        <v>-40.3052814857806</v>
       </c>
       <c r="D25" s="4" t="n">
         <f aca="false">D24-D22</f>
-        <v>-1031.24434126524</v>
+        <v>-942.244341265235</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B26" s="4" t="n">
         <f aca="false">Inputs!$B$44</f>
@@ -3555,12 +3558,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>3</v>
@@ -3574,7 +3577,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B31" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$25,Inputs!$B$26)</f>
@@ -3591,7 +3594,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B32" s="4" t="n">
         <f aca="false">2*Inputs!$B$28</f>
@@ -3608,7 +3611,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B33" s="4" t="n">
         <f aca="false">Inputs!$B$33*Inputs!$B$29</f>
@@ -3625,7 +3628,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>0</v>
@@ -3640,7 +3643,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>0</v>
@@ -3655,7 +3658,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3672,7 +3675,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B37" s="4" t="n">
         <v>0</v>
@@ -3687,7 +3690,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">Inputs!$B$46*Inputs!$B$38/Inputs!$B$7</f>
@@ -3704,7 +3707,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">Inputs!$B$46*Inputs!$B$39</f>
@@ -3721,7 +3724,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B40" s="4" t="n">
         <f aca="false">Inputs!$B$40</f>
@@ -3737,7 +3740,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B41" s="4" t="n">
         <v>0</v>
@@ -3752,7 +3755,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>0</v>
@@ -3767,7 +3770,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B43" s="4" t="n">
         <f aca="false">Inputs!$B$33*Inputs!$B$21</f>
@@ -3784,7 +3787,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B44" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -3801,7 +3804,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -3818,7 +3821,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B46" s="12" t="n">
         <f aca="false">SUM(B31:B45)</f>
@@ -3835,7 +3838,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B47" s="4" t="n">
         <f aca="false">B46-SUM(B43:B45)</f>
@@ -3852,7 +3855,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B48" s="4" t="n">
         <f aca="false">Inputs!$B$15</f>
@@ -3869,7 +3872,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B49" s="4" t="n">
         <f aca="false">B48-B46</f>
@@ -3886,24 +3889,24 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2"/>
       <c r="B53" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B54" s="10" t="n">
         <v>20</v>
@@ -3917,7 +3920,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B55" s="2" t="n">
         <f aca="false">B54-1</f>
@@ -3934,7 +3937,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B56" s="2" t="n">
         <f aca="false">INT(B55/Inputs!$B$50)</f>
@@ -3951,7 +3954,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B57" s="4" t="n">
         <f aca="false">B12+B14+B15</f>
@@ -3968,24 +3971,24 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B58" s="4" t="n">
         <f aca="false">B22</f>
-        <v>2334.24434126524</v>
+        <v>2245.24434126524</v>
       </c>
       <c r="C58" s="4" t="n">
         <f aca="false">B22</f>
-        <v>2334.24434126524</v>
+        <v>2245.24434126524</v>
       </c>
       <c r="D58" s="4" t="n">
         <f aca="false">B22</f>
-        <v>2334.24434126524</v>
+        <v>2245.24434126524</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B59" s="4" t="n">
         <f aca="false">MIN(B56,1)*B57</f>
@@ -4002,29 +4005,29 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B62" s="4" t="n">
         <f aca="false">B58-B59</f>
-        <v>1536</v>
+        <v>1447</v>
       </c>
       <c r="C62" s="4" t="n">
         <f aca="false">C58-C59</f>
-        <v>1536</v>
+        <v>1447</v>
       </c>
       <c r="D62" s="4" t="n">
         <f aca="false">D58-D59</f>
-        <v>1536</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B63" s="4" t="n">
         <v>0</v>
@@ -4038,119 +4041,119 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B65" s="5" t="n">
         <f aca="false">(B58-B59)/B55</f>
-        <v>80.8421052631579</v>
+        <v>76.1578947368421</v>
       </c>
       <c r="C65" s="5" t="n">
         <f aca="false">(C58-C59)/C55</f>
-        <v>52.9655172413793</v>
+        <v>49.8965517241379</v>
       </c>
       <c r="D65" s="5" t="n">
         <f aca="false">(D58-D59)/D55</f>
-        <v>39.3846153846154</v>
+        <v>37.1025641025641</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B66" s="4" t="n">
         <f aca="false">B22+B65</f>
-        <v>2415.08644652839</v>
+        <v>2321.40223600208</v>
       </c>
       <c r="C66" s="4" t="n">
         <f aca="false">B22+C65</f>
-        <v>2387.20985850661</v>
+        <v>2295.14089298937</v>
       </c>
       <c r="D66" s="4" t="n">
         <f aca="false">B22+D65</f>
-        <v>2373.62895664985</v>
+        <v>2282.3469053678</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B67" s="4" t="n">
         <f aca="false">C22+B65</f>
-        <v>2510.14738674894</v>
+        <v>2416.46317622262</v>
       </c>
       <c r="C67" s="4" t="n">
         <f aca="false">C22+C65</f>
-        <v>2482.27079872716</v>
+        <v>2390.20183320992</v>
       </c>
       <c r="D67" s="4" t="n">
         <f aca="false">C22+D65</f>
-        <v>2468.6898968704</v>
+        <v>2377.40784558834</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B69" s="5" t="n">
         <f aca="false">B58/B55</f>
-        <v>122.854965329749</v>
+        <v>118.170754803433</v>
       </c>
       <c r="C69" s="5" t="n">
         <f aca="false">B58/C55</f>
-        <v>80.4911841815598</v>
+        <v>77.4222186643185</v>
       </c>
       <c r="D69" s="5" t="n">
         <f aca="false">B58/D55</f>
-        <v>59.8524190068009</v>
+        <v>57.5703677247496</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B70" s="4" t="n">
         <f aca="false">B22+B69</f>
-        <v>2457.09930659498</v>
+        <v>2363.41509606867</v>
       </c>
       <c r="C70" s="4" t="n">
         <f aca="false">B22+C69</f>
-        <v>2414.7355254468</v>
+        <v>2322.66655992955</v>
       </c>
       <c r="D70" s="4" t="n">
         <f aca="false">B22+D69</f>
-        <v>2394.09676027204</v>
+        <v>2302.81470898999</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B71" s="4" t="n">
         <f aca="false">C22+B69</f>
-        <v>2552.16024681553</v>
+        <v>2458.47603628921</v>
       </c>
       <c r="C71" s="4" t="n">
         <f aca="false">C22+C69</f>
-        <v>2509.79646566734</v>
+        <v>2417.7275001501</v>
       </c>
       <c r="D71" s="4" t="n">
         <f aca="false">C22+D69</f>
-        <v>2489.15770049258</v>
+        <v>2397.87564921053</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B72" s="2" t="n">
         <f aca="false">MAX(B56-1,0)</f>
@@ -4167,26 +4170,26 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B77" s="4" t="n">
         <f aca="false">Inputs!$B$25</f>
@@ -4203,64 +4206,64 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B78" s="4" t="n">
         <f aca="false">B22-B7+B77</f>
-        <v>2218.24434126524</v>
+        <v>2129.24434126524</v>
       </c>
       <c r="C78" s="4" t="n">
         <f aca="false">B22-B7+C77</f>
-        <v>2334.24434126524</v>
+        <v>2245.24434126524</v>
       </c>
       <c r="D78" s="4" t="n">
         <f aca="false">B22-B7+D77</f>
-        <v>2450.24434126524</v>
+        <v>2361.24434126524</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">C22-B7+B77</f>
-        <v>2313.30528148578</v>
+        <v>2224.30528148578</v>
       </c>
       <c r="C79" s="4" t="n">
         <f aca="false">C22-B7+C77</f>
-        <v>2429.30528148578</v>
+        <v>2340.30528148578</v>
       </c>
       <c r="D79" s="4" t="n">
         <f aca="false">C22-B7+D77</f>
-        <v>2545.30528148578</v>
+        <v>2456.30528148578</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B22-B7+Inputs!$B$27</f>
-        <v>2050.24434126524</v>
+        <v>1961.24434126524</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B83" s="13" t="n">
         <f aca="false">Inputs!$B$7*0.9</f>
@@ -4277,7 +4280,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B84" s="14" t="n">
         <f aca="false">Inputs!$B$36+Inputs!$B$45*Inputs!$B$38</f>
@@ -4294,57 +4297,57 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B85" s="4" t="n">
         <f aca="false">B22-B12-B14+B84/B83</f>
-        <v>2409.04926807248</v>
+        <v>2320.04926807248</v>
       </c>
       <c r="C85" s="4" t="n">
         <f aca="false">B22-B12-B14+C84/C83</f>
-        <v>2334.24434126524</v>
+        <v>2245.24434126524</v>
       </c>
       <c r="D85" s="4" t="n">
         <f aca="false">B22-B12-B14+D84/D83</f>
-        <v>2273.04031024112</v>
+        <v>2184.04031024112</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B91" s="4" t="n">
         <f aca="false">B58-B57</f>
-        <v>1536</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">Inputs!$B$15-B22</f>
-        <v>-334.244341265235</v>
+        <v>-245.244341265235</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B93" s="2" t="str">
         <f aca="false">IF(B92&gt;0,ROUNDUP(B91/B92,0)+1,"not viable at this price")</f>
@@ -4353,16 +4356,16 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B94" s="4" t="n">
         <f aca="false">Inputs!$B$16-C22</f>
-        <v>-129.305281485781</v>
+        <v>-40.3052814857806</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B95" s="2" t="str">
         <f aca="false">IF(B94&gt;0,ROUNDUP(B91/B94,0)+1,"not viable at this price")</f>
@@ -4371,135 +4374,135 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C101" s="4" t="n">
         <v>600</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C102" s="4" t="n">
         <f aca="false">0.25*B12</f>
         <v>152.3505513639</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C103" s="4" t="n">
         <f aca="false">Inputs!$B$29</f>
         <v>54</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C105" s="4" t="n">
         <f aca="false">B22-600</f>
-        <v>1734.24434126524</v>
+        <v>1645.24434126524</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" s="2" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -4527,22 +4530,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>3</v>
@@ -4556,7 +4559,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$53,Inputs!$B$54)</f>
@@ -4573,7 +4576,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B8" s="4" t="n">
         <f aca="false">2*Inputs!$B$71*Inputs!$B$6</f>
@@ -4590,7 +4593,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$58*Inputs!$B$6</f>
@@ -4607,7 +4610,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
@@ -4622,7 +4625,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
@@ -4637,7 +4640,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">Inputs!$B$62*Inputs!$B$6</f>
@@ -4654,7 +4657,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>0</v>
@@ -4669,7 +4672,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
@@ -4686,7 +4689,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">(Inputs!$B$66+Inputs!$B$67)*Inputs!$B$6</f>
@@ -4703,7 +4706,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">Inputs!$B$72*Inputs!$B$6</f>
@@ -4720,7 +4723,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">Inputs!$B$73*Inputs!$B$6</f>
@@ -4737,7 +4740,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B18" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
@@ -4754,7 +4757,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -4771,7 +4774,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B20" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -4788,7 +4791,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">SUM(B7:B20)</f>
@@ -4805,7 +4808,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B22" s="4" t="n">
         <f aca="false">B21-SUM(B18:B20)</f>
@@ -4822,7 +4825,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B23" s="4" t="n">
         <f aca="false">Inputs!$B$17</f>
@@ -4839,7 +4842,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B24" s="4" t="n">
         <f aca="false">B23-B21</f>
@@ -4856,12 +4859,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>3</v>
@@ -4875,7 +4878,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$53,Inputs!$B$54)</f>
@@ -4892,7 +4895,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B30" s="4" t="n">
         <f aca="false">2*Inputs!$B$69*Inputs!$B$6</f>
@@ -4909,7 +4912,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B31" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$59*Inputs!$B$6</f>
@@ -4926,7 +4929,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>0</v>
@@ -4941,7 +4944,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>0</v>
@@ -4956,7 +4959,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B34" s="4" t="n">
         <f aca="false">Inputs!$B$62*Inputs!$B$6</f>
@@ -4973,7 +4976,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>0</v>
@@ -4988,7 +4991,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
@@ -5005,7 +5008,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B37" s="4" t="n">
         <f aca="false">(Inputs!$B$66+Inputs!$B$67)*Inputs!$B$6</f>
@@ -5022,7 +5025,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">Inputs!$B$72*Inputs!$B$6</f>
@@ -5039,7 +5042,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">Inputs!$B$73*Inputs!$B$6</f>
@@ -5056,7 +5059,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B40" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
@@ -5073,7 +5076,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B41" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -5090,7 +5093,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B42" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -5107,7 +5110,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B43" s="12" t="n">
         <f aca="false">SUM(B29:B42)</f>
@@ -5124,7 +5127,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B44" s="4" t="n">
         <f aca="false">B43-SUM(B40:B42)</f>
@@ -5141,7 +5144,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Inputs!$B$17</f>
@@ -5158,7 +5161,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B46" s="4" t="n">
         <f aca="false">B45-B43</f>
@@ -5175,7 +5178,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B47" s="4" t="n">
         <f aca="false">Inputs!$B$56</f>
@@ -5192,24 +5195,24 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2"/>
       <c r="B51" s="3" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B52" s="10" t="n">
         <v>15</v>
@@ -5223,7 +5226,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B53" s="2" t="n">
         <f aca="false">B52-1</f>
@@ -5240,7 +5243,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B54" s="2" t="n">
         <f aca="false">IF(B52&gt;=Inputs!$B$78,2,IF(B52&gt;=Inputs!$B$77,1,0))</f>
@@ -5257,7 +5260,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B55" s="4" t="n">
         <f aca="false">B9+B8+B12</f>
@@ -5274,7 +5277,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B56" s="4" t="n">
         <f aca="false">B21</f>
@@ -5291,7 +5294,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B57" s="4" t="n">
         <f aca="false">MIN(B54,1)*B55</f>
@@ -5308,12 +5311,12 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B60" s="4" t="n">
         <f aca="false">B56-B57</f>
@@ -5330,7 +5333,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B61" s="4" t="n">
         <v>0</v>
@@ -5344,12 +5347,12 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B63" s="5" t="n">
         <f aca="false">(B56-B57)/B53</f>
@@ -5366,7 +5369,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B64" s="4" t="n">
         <f aca="false">B21+B63</f>
@@ -5383,7 +5386,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B65" s="4" t="n">
         <f aca="false">C21+B63</f>
@@ -5400,12 +5403,12 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B67" s="5" t="n">
         <f aca="false">B56/B53</f>
@@ -5422,7 +5425,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B68" s="4" t="n">
         <f aca="false">B21+B67</f>
@@ -5439,7 +5442,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B69" s="4" t="n">
         <f aca="false">C21+B67</f>
@@ -5456,7 +5459,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B70" s="4" t="n">
         <v>0</v>
@@ -5471,7 +5474,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B71" s="4" t="n">
         <v>0</v>
@@ -5486,26 +5489,26 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B76" s="4" t="n">
         <f aca="false">Inputs!$B$53</f>
@@ -5522,7 +5525,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B77" s="4" t="n">
         <f aca="false">B21-B7+B76</f>
@@ -5539,7 +5542,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B78" s="4" t="n">
         <f aca="false">C21-B7+B76</f>
@@ -5556,7 +5559,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">D21-B7+B76</f>
@@ -5573,7 +5576,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B21-B7+Inputs!$B$55-B8+2*Inputs!$B$69*Inputs!$B$6</f>
@@ -5582,21 +5585,21 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B83" s="15" t="n">
         <f aca="false">Inputs!$B$6*0.9</f>
@@ -5613,7 +5616,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B84" s="4" t="n">
         <f aca="false">(B7+B18+B19+B20)+(B21-(B7+B18+B19+B20))*B83/Inputs!$B$6</f>
@@ -5630,7 +5633,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B85" s="4" t="n">
         <f aca="false">(C7+C18+C19+C20)+(C21-(C7+C18+C19+C20))*B83/Inputs!$B$6</f>
@@ -5647,12 +5650,12 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B89" s="4" t="n">
         <f aca="false">B56-B55</f>
@@ -5661,7 +5664,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B90" s="4" t="n">
         <f aca="false">Inputs!$B$17-B21</f>
@@ -5670,7 +5673,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B91" s="2" t="n">
         <f aca="false">IF(B90&gt;0,ROUNDUP(B89/B90,0)+1,"not viable at this price")</f>
@@ -5679,7 +5682,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">Inputs!$B$17-C21</f>
@@ -5688,7 +5691,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B93" s="2" t="str">
         <f aca="false">IF(B92&gt;0,ROUNDUP(B89/B92,0)+1,"not viable at this price")</f>
@@ -5697,106 +5700,106 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C99" s="4" t="n">
         <v>700</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C100" s="4" t="n">
         <f aca="false">0.5*(B9+B8+B12)</f>
         <v>514.20525</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C102" s="4" t="n">
         <f aca="false">B21-700</f>
         <v>1877.475</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
       <c r="D104" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -5824,17 +5827,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>8</v>
@@ -5848,26 +5851,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$81,Inputs!$B$82)</f>
@@ -5884,7 +5887,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B10" s="4" t="n">
         <f aca="false">(ROUNDUP(B5/Inputs!$B$94,0)*(Inputs!$B$83*Inputs!$B$93+Inputs!$B$95))/B5</f>
@@ -5901,7 +5904,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B11" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$85</f>
@@ -5918,7 +5921,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">(Inputs!$B$89-Inputs!$B$91)*Inputs!$B$87</f>
@@ -5935,7 +5938,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B13" s="4" t="n">
         <f aca="false">Inputs!$B$91*Inputs!$B$88</f>
@@ -5952,7 +5955,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">Inputs!$B$92</f>
@@ -5969,7 +5972,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$21</f>
@@ -5986,7 +5989,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6003,7 +6006,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6020,7 +6023,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">SUM(B9:B17)</f>
@@ -6037,7 +6040,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">B18-SUM(B15:B17)</f>
@@ -6054,7 +6057,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B20" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6071,7 +6074,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B21" s="4" t="n">
         <f aca="false">B20-B18</f>
@@ -6088,26 +6091,26 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B26" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$81,Inputs!$B$82)</f>
@@ -6124,7 +6127,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">(ROUNDUP(B5/Inputs!$B$94,0)*(Inputs!$B$84*Inputs!$B$93+Inputs!$B$95))/B5</f>
@@ -6141,7 +6144,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$85</f>
@@ -6158,7 +6161,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">(Inputs!$B$90-Inputs!$B$91)*Inputs!$B$87</f>
@@ -6175,7 +6178,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B30" s="4" t="n">
         <f aca="false">Inputs!$B$91*Inputs!$B$88</f>
@@ -6192,7 +6195,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B31" s="4" t="n">
         <f aca="false">Inputs!$B$92</f>
@@ -6209,7 +6212,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B32" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$21</f>
@@ -6226,7 +6229,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B33" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6243,7 +6246,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B34" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6260,7 +6263,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B35" s="12" t="n">
         <f aca="false">SUM(B26:B34)</f>
@@ -6277,7 +6280,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">B35-SUM(B32:B34)</f>
@@ -6294,7 +6297,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B37" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6311,7 +6314,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">B37-B35</f>
@@ -6328,26 +6331,26 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B43" s="4" t="n">
         <f aca="false">Inputs!$B$100+Inputs!$B$101</f>
@@ -6364,7 +6367,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B44" s="4" t="n">
         <f aca="false">Inputs!$B$105</f>
@@ -6381,7 +6384,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$103</f>
@@ -6398,7 +6401,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B46" s="4" t="n">
         <f aca="false">Inputs!$B$98*Inputs!$B$96*(1+Inputs!$B$97)</f>
@@ -6415,7 +6418,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B47" s="4" t="n">
         <f aca="false">Inputs!$B$98*Inputs!$B$106</f>
@@ -6432,7 +6435,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B48" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$21</f>
@@ -6449,7 +6452,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B49" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6466,7 +6469,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B50" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6483,7 +6486,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B51" s="12" t="n">
         <f aca="false">SUM(B43:B50)</f>
@@ -6500,7 +6503,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B52" s="4" t="n">
         <f aca="false">B51-SUM(B48:B50)</f>
@@ -6517,7 +6520,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B53" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6534,7 +6537,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B54" s="4" t="n">
         <f aca="false">B53-B51</f>
@@ -6551,7 +6554,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B55" s="12" t="n">
         <f aca="false">B51-B18</f>
@@ -6568,7 +6571,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B56" s="4" t="n">
         <f aca="false">Inputs!$B$101-Inputs!$B$102</f>
@@ -6585,26 +6588,26 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B61" s="4" t="n">
         <f aca="false">Inputs!$B$100+Inputs!$B$101</f>
@@ -6621,7 +6624,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B62" s="4" t="n">
         <f aca="false">Inputs!$B$105</f>
@@ -6638,7 +6641,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B63" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$103</f>
@@ -6655,7 +6658,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B64" s="4" t="n">
         <f aca="false">Inputs!$B$99*Inputs!$B$96*(1+Inputs!$B$97)</f>
@@ -6672,7 +6675,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B65" s="4" t="n">
         <f aca="false">Inputs!$B$99*Inputs!$B$106</f>
@@ -6689,7 +6692,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B66" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$21</f>
@@ -6706,7 +6709,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B67" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6723,7 +6726,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B68" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6740,7 +6743,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B69" s="12" t="n">
         <f aca="false">SUM(B61:B68)</f>
@@ -6757,7 +6760,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B70" s="4" t="n">
         <f aca="false">B69-SUM(B66:B68)</f>
@@ -6774,7 +6777,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B71" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6791,7 +6794,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B72" s="4" t="n">
         <f aca="false">B71-B69</f>
@@ -6808,7 +6811,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B73" s="12" t="n">
         <f aca="false">B69-B35</f>
@@ -6825,17 +6828,17 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B78" s="2" t="n">
         <f aca="false">B5-1</f>
@@ -6852,7 +6855,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">B12+B13</f>
@@ -6869,7 +6872,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B18</f>
@@ -6886,7 +6889,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B81" s="4" t="n">
         <f aca="false">B80-B79</f>
@@ -6903,7 +6906,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B82" s="5" t="n">
         <f aca="false">(B80-B79)/B78</f>
@@ -6920,7 +6923,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B83" s="5" t="n">
         <f aca="false">B80/B78</f>
@@ -6937,7 +6940,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B84" s="4" t="n">
         <f aca="false">B18+B83</f>
@@ -6954,26 +6957,26 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B89" s="4" t="n">
         <f aca="false">Inputs!$B$81</f>
@@ -6990,7 +6993,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B90" s="4" t="n">
         <f aca="false">C18-C9+B89</f>
@@ -7007,7 +7010,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B91" s="4" t="n">
         <f aca="false">C18-C13+Inputs!$B$87</f>
@@ -7016,7 +7019,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">C18-Inputs!$B$83*(Inputs!$B$85-Inputs!$B$86)</f>
@@ -7025,12 +7028,12 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B96" s="4" t="n">
         <f aca="false">Inputs!$B$14-C18</f>
@@ -7039,7 +7042,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B97" s="2" t="str">
         <f aca="false">IF(B96&gt;0,ROUNDUP(C80/B96,0)+1,"not viable at this price")</f>
@@ -7048,120 +7051,120 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C104" s="4" t="n">
         <v>400</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C105" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$81,Inputs!$B$82)</f>
         <v>550</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C106" s="4" t="n">
         <f aca="false">Inputs!$B$85</f>
         <v>75</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C107" s="4" t="n">
         <f aca="false">0.25*(C12+C13)</f>
         <v>97.5</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C108" s="4" t="n">
         <f aca="false">C18-400</f>
         <v>1296</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C109" s="4" t="n">
         <f aca="false">Inputs!$B$98*Inputs!$B$96*(1+Inputs!$B$97)</f>
         <v>877.8</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Process first replies: quoted inputs, suggested-reply drafts, tracker update
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/december_pricing.xlsx
+++ b/december-plan/pricing/december_pricing.xlsx
@@ -230,10 +230,10 @@
     <t xml:space="preserve">Nights, 5-night version</t>
   </si>
   <si>
-    <t xml:space="preserve">PADI Open Water in-water course, gear incl. (Blue Note)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED (snippet); second snippet shows USD 300</t>
+    <t xml:space="preserve">PADI Open Water in-water course, gear, wetsuit and DAN training cover incl. (Sand Dollar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-22 (Sand Dollar email); Blue Note advertised 400</t>
   </si>
   <si>
     <t xml:space="preserve">PADI Open Water eLearning, bought from PADI</t>
@@ -251,10 +251,10 @@
     <t xml:space="preserve">ADVERTISED (snippet); USD 600 listed</t>
   </si>
   <si>
-    <t xml:space="preserve">Two-tank boat dive, mid of island band</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED (snippet); 95–135</t>
+    <t xml:space="preserve">Two-tank boat dive incl. steel tanks and weights (Aldora)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-22 (Aldora email)</t>
   </si>
   <si>
     <t xml:space="preserve">Marine park fee per dive day</t>
@@ -278,10 +278,7 @@
     <t xml:space="preserve">ADVERTISED (snippet); Salty USD 350 + IVA</t>
   </si>
   <si>
-    <t xml:space="preserve">Nitrox fill per tank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED (snippet); 10–13</t>
+    <t xml:space="preserve">Nitrox fill per tank (Aldora)</t>
   </si>
   <si>
     <t xml:space="preserve">Night dive, 1 tank</t>
@@ -323,7 +320,7 @@
     <t xml:space="preserve">paying</t>
   </si>
   <si>
-    <t xml:space="preserve">QUOTE NEEDED; brief convention</t>
+    <t xml:space="preserve">QUOTED 2026-09-22: Aldora 1 comp at 10+ paid; Sand Dollar one free diver</t>
   </si>
   <si>
     <t xml:space="preserve">Egypt (Marsa Shagra), Sat 2 – Sat 9 Jan 2027, 6 nights on the ground</t>
@@ -464,7 +461,10 @@
     <t xml:space="preserve">La Parguera hotel, pp/night, 3 sharing</t>
   </si>
   <si>
-    <t xml:space="preserve">Two-tank Wall dive, gear included (Paradise Scuba)</t>
+    <t xml:space="preserve">Two-tank Wall dive (Paradise Scuba): USD 145 less 15% group discount, plus 11.5% tax; own gear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-22 price and discount; tax rate INFERRED (PR IVU), QUOTE NEEDED</t>
   </si>
   <si>
     <t xml:space="preserve">Desecheo two-tank incl. USD 20 park fee (Taino Divers), own gear</t>
@@ -482,7 +482,7 @@
     <t xml:space="preserve">Of which Desecheo days (weather permitting)</t>
   </si>
   <si>
-    <t xml:space="preserve">Bio bay boat tour (Parguera Eco Tours)</t>
+    <t xml:space="preserve">Bio bay boat tour (Parguera Eco Tours; Paradise Scuba also offers, price pending)</t>
   </si>
   <si>
     <t xml:space="preserve">Car hire per car per day (mid-size, SJU)</t>
@@ -1546,11 +1546,11 @@
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Cozumel!C22</f>
-        <v>2340.30528148578</v>
+        <v>2270.30528148578</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">Cozumel!D22</f>
-        <v>2942.24434126524</v>
+        <v>2936.24434126524</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1580,11 +1580,11 @@
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">C8-C7</f>
-        <v>-40.3052814857806</v>
+        <v>29.6947185142194</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">D8-D7</f>
-        <v>-942.244341265235</v>
+        <v>-936.244341265235</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1614,11 +1614,11 @@
       </c>
       <c r="C11" s="4" t="n">
         <f aca="false">Cozumel!C46</f>
-        <v>2093.53685432385</v>
+        <v>2033.53685432385</v>
       </c>
       <c r="D11" s="4" t="n">
         <f aca="false">Cozumel!D46</f>
-        <v>2815.47591410331</v>
+        <v>2809.47591410331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1631,11 +1631,11 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">Cozumel!C23</f>
-        <v>1961.30528148578</v>
+        <v>1891.30528148578</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">Cozumel!D23</f>
-        <v>2563.24434126524</v>
+        <v>2557.24434126524</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1777,11 +1777,11 @@
       </c>
       <c r="B25" s="4" t="n">
         <f aca="false">Thanksgiving!C18</f>
-        <v>1696</v>
+        <v>1720</v>
       </c>
       <c r="C25" s="4" t="n">
         <f aca="false">Thanksgiving!C35</f>
-        <v>1952</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1816,11 +1816,11 @@
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">B27-B25</f>
-        <v>-196</v>
+        <v>-220</v>
       </c>
       <c r="C28" s="4" t="n">
         <f aca="false">C27-C25</f>
-        <v>-452</v>
+        <v>-488</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">B26-B25</f>
-        <v>670.8</v>
+        <v>646.8</v>
       </c>
       <c r="C29" s="4" t="n">
         <f aca="false">C26-C25</f>
-        <v>1028.7</v>
+        <v>992.7</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1842,11 +1842,11 @@
       </c>
       <c r="B30" s="4" t="n">
         <f aca="false">Thanksgiving!C19</f>
-        <v>1387</v>
+        <v>1411</v>
       </c>
       <c r="C30" s="4" t="n">
         <f aca="false">Thanksgiving!C36</f>
-        <v>1608</v>
+        <v>1644</v>
       </c>
     </row>
   </sheetData>
@@ -2194,7 +2194,7 @@
         <v>68</v>
       </c>
       <c r="B34" s="9" t="n">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>41</v>
@@ -2236,7 +2236,7 @@
         <v>75</v>
       </c>
       <c r="B37" s="9" t="n">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>41</v>
@@ -2306,18 +2306,18 @@
         <v>84</v>
       </c>
       <c r="B42" s="9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B43" s="9" t="n">
         <v>95</v>
@@ -2331,7 +2331,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B44" s="9" t="n">
         <v>260</v>
@@ -2340,74 +2340,74 @@
         <v>41</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B45" s="10" t="n">
         <v>5</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D45" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B46" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B47" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C47" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D47" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B48" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C48" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B49" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>31</v>
@@ -2415,26 +2415,26 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B50" s="10" t="n">
         <v>10</v>
       </c>
       <c r="C50" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D50" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B53" s="9" t="n">
         <v>700</v>
@@ -2448,7 +2448,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B54" s="9" t="n">
         <v>1300</v>
@@ -2462,7 +2462,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B55" s="9" t="n">
         <v>1300</v>
@@ -2471,12 +2471,12 @@
         <v>41</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B56" s="9" t="n">
         <v>0</v>
@@ -2485,12 +2485,12 @@
         <v>41</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B57" s="10" t="n">
         <v>6</v>
@@ -2499,228 +2499,228 @@
         <v>65</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B58" s="11" t="n">
         <v>78</v>
       </c>
       <c r="C58" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D58" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B59" s="11" t="n">
         <v>113</v>
       </c>
       <c r="C59" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D59" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="D59" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B60" s="11" t="n">
         <v>358</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B61" s="11" t="n">
         <v>94</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B62" s="11" t="n">
         <v>347</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B63" s="11" t="n">
         <v>69</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B64" s="11" t="n">
         <v>15</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B65" s="11" t="n">
         <v>315</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B66" s="11" t="n">
         <v>67</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B67" s="11" t="n">
         <v>59</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B68" s="11" t="n">
         <v>80</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B69" s="11" t="n">
         <v>22</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B70" s="11" t="n">
         <v>17</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B71" s="11" t="n">
         <v>41</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B72" s="11" t="n">
         <v>45</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B73" s="11" t="n">
         <v>7</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>31</v>
@@ -2728,7 +2728,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B74" s="9" t="n">
         <v>15</v>
@@ -2742,41 +2742,41 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B75" s="10" t="n">
         <v>5</v>
       </c>
       <c r="C75" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D75" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D75" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B76" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C76" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D76" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B77" s="10" t="n">
         <v>11</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>31</v>
@@ -2784,26 +2784,26 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B78" s="10" t="n">
         <v>22</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B81" s="9" t="n">
         <v>400</v>
@@ -2812,12 +2812,12 @@
         <v>41</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B82" s="9" t="n">
         <v>700</v>
@@ -2826,12 +2826,12 @@
         <v>41</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B83" s="10" t="n">
         <v>4</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B84" s="10" t="n">
         <v>5</v>
@@ -2859,7 +2859,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B85" s="9" t="n">
         <v>75</v>
@@ -2873,7 +2873,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B86" s="9" t="n">
         <v>50</v>
@@ -2887,16 +2887,16 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B87" s="9" t="n">
-        <v>125</v>
+        <v>137</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>31</v>
+        <v>146</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2921,10 +2921,10 @@
         <v>3</v>
       </c>
       <c r="C89" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D89" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2935,10 +2935,10 @@
         <v>4</v>
       </c>
       <c r="C90" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D90" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D90" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2949,10 +2949,10 @@
         <v>1</v>
       </c>
       <c r="C91" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D91" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D91" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2980,7 +2980,7 @@
         <v>41</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3047,10 +3047,10 @@
         <v>2</v>
       </c>
       <c r="C98" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D98" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3061,10 +3061,10 @@
         <v>3</v>
       </c>
       <c r="C99" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D99" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D99" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3078,7 +3078,7 @@
         <v>41</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3148,7 +3148,7 @@
         <v>41</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="C10" s="4" t="n">
         <f aca="false">Inputs!$B$34</f>
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>0</v>
@@ -3318,7 +3318,7 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">Inputs!$B$47*Inputs!$B$37</f>
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3402,7 +3402,7 @@
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">6*Inputs!$B$42</f>
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3481,11 +3481,11 @@
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">SUM(C7:C21)</f>
-        <v>2340.30528148578</v>
+        <v>2270.30528148578</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">SUM(D7:D21)</f>
-        <v>2942.24434126524</v>
+        <v>2936.24434126524</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3498,11 +3498,11 @@
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">C22-SUM(C19:C21)</f>
-        <v>1961.30528148578</v>
+        <v>1891.30528148578</v>
       </c>
       <c r="D23" s="4" t="n">
         <f aca="false">D22-SUM(D19:D21)</f>
-        <v>2563.24434126524</v>
+        <v>2557.24434126524</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3532,11 +3532,11 @@
       </c>
       <c r="C25" s="4" t="n">
         <f aca="false">C24-C22</f>
-        <v>-40.3052814857806</v>
+        <v>29.6947185142194</v>
       </c>
       <c r="D25" s="4" t="n">
         <f aca="false">D24-D22</f>
-        <v>-942.244341265235</v>
+        <v>-936.244341265235</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="C34" s="4" t="n">
         <f aca="false">Inputs!$B$34</f>
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="D34" s="4" t="n">
         <v>0</v>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C36" s="4" t="n">
         <f aca="false">Inputs!$B$48*Inputs!$B$37</f>
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="D36" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="D41" s="4" t="n">
         <f aca="false">6*Inputs!$B$42</f>
-        <v>72</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3829,11 +3829,11 @@
       </c>
       <c r="C46" s="12" t="n">
         <f aca="false">SUM(C31:C45)</f>
-        <v>2093.53685432385</v>
+        <v>2033.53685432385</v>
       </c>
       <c r="D46" s="12" t="n">
         <f aca="false">SUM(D31:D45)</f>
-        <v>2815.47591410331</v>
+        <v>2809.47591410331</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3846,11 +3846,11 @@
       </c>
       <c r="C47" s="4" t="n">
         <f aca="false">C46-SUM(C43:C45)</f>
-        <v>1749.53685432385</v>
+        <v>1689.53685432385</v>
       </c>
       <c r="D47" s="4" t="n">
         <f aca="false">D46-SUM(D43:D45)</f>
-        <v>2471.47591410331</v>
+        <v>2465.47591410331</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3880,11 +3880,11 @@
       </c>
       <c r="C49" s="4" t="n">
         <f aca="false">C48-C46</f>
-        <v>206.463145676146</v>
+        <v>266.463145676146</v>
       </c>
       <c r="D49" s="4" t="n">
         <f aca="false">D48-D46</f>
-        <v>-815.475914103308</v>
+        <v>-809.475914103308</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4084,15 +4084,15 @@
       </c>
       <c r="B67" s="4" t="n">
         <f aca="false">C22+B65</f>
-        <v>2416.46317622262</v>
+        <v>2346.46317622262</v>
       </c>
       <c r="C67" s="4" t="n">
         <f aca="false">C22+C65</f>
-        <v>2390.20183320992</v>
+        <v>2320.20183320992</v>
       </c>
       <c r="D67" s="4" t="n">
         <f aca="false">C22+D65</f>
-        <v>2377.40784558834</v>
+        <v>2307.40784558834</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4140,15 +4140,15 @@
       </c>
       <c r="B71" s="4" t="n">
         <f aca="false">C22+B69</f>
-        <v>2458.47603628921</v>
+        <v>2388.47603628921</v>
       </c>
       <c r="C71" s="4" t="n">
         <f aca="false">C22+C69</f>
-        <v>2417.7275001501</v>
+        <v>2347.7275001501</v>
       </c>
       <c r="D71" s="4" t="n">
         <f aca="false">C22+D69</f>
-        <v>2397.87564921053</v>
+        <v>2327.87564921053</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4227,15 +4227,15 @@
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">C22-B7+B77</f>
-        <v>2224.30528148578</v>
+        <v>2154.30528148578</v>
       </c>
       <c r="C79" s="4" t="n">
         <f aca="false">C22-B7+C77</f>
-        <v>2340.30528148578</v>
+        <v>2270.30528148578</v>
       </c>
       <c r="D79" s="4" t="n">
         <f aca="false">C22-B7+D77</f>
-        <v>2456.30528148578</v>
+        <v>2386.30528148578</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4360,16 +4360,16 @@
       </c>
       <c r="B94" s="4" t="n">
         <f aca="false">Inputs!$B$16-C22</f>
-        <v>-40.3052814857806</v>
+        <v>29.6947185142194</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="B95" s="2" t="str">
+      <c r="B95" s="2" t="n">
         <f aca="false">IF(B94&gt;0,ROUNDUP(B91/B94,0)+1,"not viable at this price")</f>
-        <v>not viable at this price</v>
+        <v>50</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4723,7 +4723,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">Inputs!$B$73*Inputs!$B$6</f>
@@ -5042,7 +5042,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">Inputs!$B$73*Inputs!$B$6</f>
@@ -5925,15 +5925,15 @@
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">(Inputs!$B$89-Inputs!$B$91)*Inputs!$B$87</f>
-        <v>250</v>
+        <v>274</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">(Inputs!$B$89-Inputs!$B$91)*Inputs!$B$87</f>
-        <v>250</v>
+        <v>274</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">(Inputs!$B$89-Inputs!$B$91)*Inputs!$B$87</f>
-        <v>250</v>
+        <v>274</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6027,15 +6027,15 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">SUM(B9:B17)</f>
-        <v>1679</v>
+        <v>1703</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">SUM(C9:C17)</f>
-        <v>1696</v>
+        <v>1720</v>
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">SUM(D9:D17)</f>
-        <v>1679</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6044,15 +6044,15 @@
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">B18-SUM(B15:B17)</f>
-        <v>1370</v>
+        <v>1394</v>
       </c>
       <c r="C19" s="4" t="n">
         <f aca="false">C18-SUM(C15:C17)</f>
-        <v>1387</v>
+        <v>1411</v>
       </c>
       <c r="D19" s="4" t="n">
         <f aca="false">D18-SUM(D15:D17)</f>
-        <v>1370</v>
+        <v>1394</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6078,15 +6078,15 @@
       </c>
       <c r="B21" s="4" t="n">
         <f aca="false">B20-B18</f>
-        <v>-179</v>
+        <v>-203</v>
       </c>
       <c r="C21" s="4" t="n">
         <f aca="false">C20-C18</f>
-        <v>-196</v>
+        <v>-220</v>
       </c>
       <c r="D21" s="4" t="n">
         <f aca="false">D20-D18</f>
-        <v>-179</v>
+        <v>-203</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6165,15 +6165,15 @@
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">(Inputs!$B$90-Inputs!$B$91)*Inputs!$B$87</f>
-        <v>375</v>
+        <v>411</v>
       </c>
       <c r="C29" s="4" t="n">
         <f aca="false">(Inputs!$B$90-Inputs!$B$91)*Inputs!$B$87</f>
-        <v>375</v>
+        <v>411</v>
       </c>
       <c r="D29" s="4" t="n">
         <f aca="false">(Inputs!$B$90-Inputs!$B$91)*Inputs!$B$87</f>
-        <v>375</v>
+        <v>411</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6267,15 +6267,15 @@
       </c>
       <c r="B35" s="12" t="n">
         <f aca="false">SUM(B26:B34)</f>
-        <v>1931.5</v>
+        <v>1967.5</v>
       </c>
       <c r="C35" s="12" t="n">
         <f aca="false">SUM(C26:C34)</f>
-        <v>1952</v>
+        <v>1988</v>
       </c>
       <c r="D35" s="12" t="n">
         <f aca="false">SUM(D26:D34)</f>
-        <v>1931.5</v>
+        <v>1967.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6284,15 +6284,15 @@
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">B35-SUM(B32:B34)</f>
-        <v>1587.5</v>
+        <v>1623.5</v>
       </c>
       <c r="C36" s="4" t="n">
         <f aca="false">C35-SUM(C32:C34)</f>
-        <v>1608</v>
+        <v>1644</v>
       </c>
       <c r="D36" s="4" t="n">
         <f aca="false">D35-SUM(D32:D34)</f>
-        <v>1587.5</v>
+        <v>1623.5</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6318,15 +6318,15 @@
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">B37-B35</f>
-        <v>-431.5</v>
+        <v>-467.5</v>
       </c>
       <c r="C38" s="4" t="n">
         <f aca="false">C37-C35</f>
-        <v>-452</v>
+        <v>-488</v>
       </c>
       <c r="D38" s="4" t="n">
         <f aca="false">D37-D35</f>
-        <v>-431.5</v>
+        <v>-467.5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6558,15 +6558,15 @@
       </c>
       <c r="B55" s="12" t="n">
         <f aca="false">B51-B18</f>
-        <v>687.8</v>
+        <v>663.8</v>
       </c>
       <c r="C55" s="12" t="n">
         <f aca="false">C51-C18</f>
-        <v>670.8</v>
+        <v>646.8</v>
       </c>
       <c r="D55" s="12" t="n">
         <f aca="false">D51-D18</f>
-        <v>687.8</v>
+        <v>663.8</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6815,15 +6815,15 @@
       </c>
       <c r="B73" s="12" t="n">
         <f aca="false">B69-B35</f>
-        <v>1049.2</v>
+        <v>1013.2</v>
       </c>
       <c r="C73" s="12" t="n">
         <f aca="false">C69-C35</f>
-        <v>1028.7</v>
+        <v>992.7</v>
       </c>
       <c r="D73" s="12" t="n">
         <f aca="false">D69-D35</f>
-        <v>1049.2</v>
+        <v>1013.2</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6859,15 +6859,15 @@
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">B12+B13</f>
-        <v>390</v>
+        <v>414</v>
       </c>
       <c r="C79" s="4" t="n">
         <f aca="false">C12+C13</f>
-        <v>390</v>
+        <v>414</v>
       </c>
       <c r="D79" s="4" t="n">
         <f aca="false">D12+D13</f>
-        <v>390</v>
+        <v>414</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6876,15 +6876,15 @@
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B18</f>
-        <v>1679</v>
+        <v>1703</v>
       </c>
       <c r="C80" s="4" t="n">
         <f aca="false">C18</f>
-        <v>1696</v>
+        <v>1720</v>
       </c>
       <c r="D80" s="4" t="n">
         <f aca="false">D18</f>
-        <v>1679</v>
+        <v>1703</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6927,15 +6927,15 @@
       </c>
       <c r="B83" s="5" t="n">
         <f aca="false">B80/B78</f>
-        <v>239.857142857143</v>
+        <v>243.285714285714</v>
       </c>
       <c r="C83" s="5" t="n">
         <f aca="false">C80/C78</f>
-        <v>188.444444444444</v>
+        <v>191.111111111111</v>
       </c>
       <c r="D83" s="5" t="n">
         <f aca="false">D80/D78</f>
-        <v>152.636363636364</v>
+        <v>154.818181818182</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6944,15 +6944,15 @@
       </c>
       <c r="B84" s="4" t="n">
         <f aca="false">B18+B83</f>
-        <v>1918.85714285714</v>
+        <v>1946.28571428571</v>
       </c>
       <c r="C84" s="4" t="n">
         <f aca="false">C18+C83</f>
-        <v>1884.44444444444</v>
+        <v>1911.11111111111</v>
       </c>
       <c r="D84" s="4" t="n">
         <f aca="false">D18+D83</f>
-        <v>1831.63636363636</v>
+        <v>1857.81818181818</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6997,15 +6997,15 @@
       </c>
       <c r="B90" s="4" t="n">
         <f aca="false">C18-C9+B89</f>
-        <v>1546</v>
+        <v>1570</v>
       </c>
       <c r="C90" s="4" t="n">
         <f aca="false">C18-C9+C89</f>
-        <v>1696</v>
+        <v>1720</v>
       </c>
       <c r="D90" s="4" t="n">
         <f aca="false">C18-C9+D89</f>
-        <v>1846</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7014,7 +7014,7 @@
       </c>
       <c r="B91" s="4" t="n">
         <f aca="false">C18-C13+Inputs!$B$87</f>
-        <v>1681</v>
+        <v>1717</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7023,7 +7023,7 @@
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">C18-Inputs!$B$83*(Inputs!$B$85-Inputs!$B$86)</f>
-        <v>1596</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7037,7 +7037,7 @@
       </c>
       <c r="B96" s="4" t="n">
         <f aca="false">Inputs!$B$14-C18</f>
-        <v>-196</v>
+        <v>-220</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7131,7 +7131,7 @@
       </c>
       <c r="C107" s="4" t="n">
         <f aca="false">0.25*(C12+C13)</f>
-        <v>97.5</v>
+        <v>103.5</v>
       </c>
       <c r="D107" s="2" t="s">
         <v>366</v>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="C108" s="4" t="n">
         <f aca="false">C18-400</f>
-        <v>1296</v>
+        <v>1320</v>
       </c>
       <c r="D108" s="2" t="s">
         <v>367</v>

</xml_diff>

<commit_message>
Cozumel dates confirmed Sun 13 – Sat 19 Dec: relabel tracker, memo, plan, workbook, flights; add date-change note for existing contacts
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/december_pricing.xlsx
+++ b/december-plan/pricing/december_pricing.xlsx
@@ -32,7 +32,7 @@
     <t xml:space="preserve">Prices before any organiser charge, at the airfare midpoint and 2 sharing. Organiser charge under Approach 2 shown separately. Every price rests on advertised or inferred figures; none is a quote.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cozumel, 6 nights (Tue 8 – Mon 14 Dec)</t>
+    <t xml:space="preserve">Cozumel, 6 nights (Sun 13 – Sat 19 Dec)</t>
   </si>
   <si>
     <t xml:space="preserve">Certified</t>
@@ -179,7 +179,7 @@
     <t xml:space="preserve">Tips and local extras per trip</t>
   </si>
   <si>
-    <t xml:space="preserve">Cozumel, Tue 8 – Mon 14 Dec 2026 (6 nights) and Tue 8 – Sun 13 Dec (5 nights)</t>
+    <t xml:space="preserve">Cozumel, Sun 13 – Sat 19 Dec 2026 (6 nights, confirmed 22 Sep) and 5-night variant</t>
   </si>
   <si>
     <t xml:space="preserve">Flight PHL–CZM return, low</t>
@@ -218,13 +218,13 @@
     <t xml:space="preserve">ADVERTISED (snippet); upper of 65–84</t>
   </si>
   <si>
-    <t xml:space="preserve">Nights, 6-night version (Tue 8 – Mon 14)</t>
+    <t xml:space="preserve">Nights, 6-night version (Sun 13 – Sat 19)</t>
   </si>
   <si>
     <t xml:space="preserve">nights</t>
   </si>
   <si>
-    <t xml:space="preserve">scope change 22 Sep</t>
+    <t xml:space="preserve">dates confirmed 22 Sep</t>
   </si>
   <si>
     <t xml:space="preserve">Nights, 5-night version</t>
@@ -557,7 +557,7 @@
     <t xml:space="preserve">George is costed as a diving participant. Free places from operators are applied first; any remainder is shown as a disclosed per-head charge.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cozumel — Tue 8 – Mon 14 Dec 2026 (6 nights) and Tue 8 – Sun 13 Dec (5 nights)</t>
+    <t xml:space="preserve">Cozumel — Sun 13 – Sat 19 Dec 2026 (6 nights, confirmed 22 Sep) and 5-night variant</t>
   </si>
   <si>
     <t xml:space="preserve">All figures per person, USD. Reads from Inputs. Lodging at Hotel Cozumel &amp; Resort, 2 sharing, breakfast included. Flights at the midpoint of the aggregator band.</t>

</xml_diff>

<commit_message>
Morning run 23 Sep: date-change notes sent, four replies processed, Sand Dollar quoted figures into the workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/december_pricing.xlsx
+++ b/december-plan/pricing/december_pricing.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="678" uniqueCount="374">
   <si>
     <t xml:space="preserve">Summary — all-in price per person vs ceiling</t>
   </si>
@@ -251,37 +251,46 @@
     <t xml:space="preserve">ADVERTISED (snippet); USD 600 listed</t>
   </si>
   <si>
-    <t xml:space="preserve">Two-tank boat dive incl. steel tanks and weights (Aldora)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED 2026-09-22 (Aldora email)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marine park fee per dive day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED (snippet); USD 15</t>
+    <t xml:space="preserve">Two-tank boat dive per day, 5-day package basis (Sand Dollar USD 510 / 5); Aldora USD 110 + tax, or 145 incl. tax and park fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-23 (Sand Dollar email: 2-day 215, 3-day 321, 4-day 420, 5-day 510); Aldora QUOTED 2026-09-22/23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marine park fee per boat day (Sand Dollar charges USD 14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-22 (Sand Dollar: USD 14/boat day, = MXN 241 at 17.23)</t>
   </si>
   <si>
     <t xml:space="preserve">Gear rental per day (certified divers)</t>
   </si>
   <si>
-    <t xml:space="preserve">Refresher (certified divers, if &gt;12 months)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brief lead; island range 30–107</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PADI Advanced Open Water incl. eLearning (Blue Note)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED (snippet); Salty USD 350 + IVA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nitrox fill per tank (Aldora)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Night dive, 1 tank</t>
+    <t xml:space="preserve">QUOTED 2026-09-22 (Aldora USD 20/day); island advertised 25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refresher / tune-up shore dive on arrival day (Sand Dollar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-23 (Sand Dollar: scuba tune-up USD 5; guided shore dive USD 5 with a package)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PADI Advanced Open Water incl. eLearning (Blue Note advertised 530; Sand Dollar QUOTED 380 in-water with eLearning done + PADI AOW eLearning bought separately; Aldora QUOTED 749 all-in)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED (snippet) kept as the conservative figure; Sand Dollar 380 + eLearning QUOTE NEEDED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nitrox fill per tank (Sand Dollar 13, about 20 tanks; Aldora 11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-23 (Sand Dollar) and 2026-09-22 (Aldora)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Night dive from the boat (Sand Dollar; shore version USD 60 incl. light)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 2026-09-23 (Sand Dollar); Aldora 82 air / 94 nitrox</t>
   </si>
   <si>
     <t xml:space="preserve">Optional bull-shark day, Playa del Carmen (BAITED), all-in incl. ferry and gear</t>
@@ -467,10 +476,10 @@
     <t xml:space="preserve">QUOTED 2026-09-22 price and discount; tax rate INFERRED (PR IVU), QUOTE NEEDED</t>
   </si>
   <si>
-    <t xml:space="preserve">Desecheo two-tank incl. USD 20 park fee (Taino Divers), own gear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADVERTISED (snippet, aggregator lead)</t>
+    <t xml:space="preserve">Desecheo two-tank incl. USD 20 park fee, own gear (Taino Divers has no boat as of 2026-09-23; Island Style Charters, max 4 divers per charter, is the referral)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADVERTISED (snippet, aggregator lead); QUOTE NEEDED</t>
   </si>
   <si>
     <t xml:space="preserve">Dive days, 25–29 Nov (Thu–Sat; Sat last dive by noon)</t>
@@ -1542,15 +1551,15 @@
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">Cozumel!B22</f>
-        <v>2245.24434126524</v>
+        <v>2201.33836331979</v>
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Cozumel!C22</f>
-        <v>2270.30528148578</v>
+        <v>2247.96169471851</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">Cozumel!D22</f>
-        <v>2936.24434126524</v>
+        <v>2894.33836331979</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1576,15 +1585,15 @@
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">B8-B7</f>
-        <v>-245.244341265235</v>
+        <v>-201.338363319791</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">C8-C7</f>
-        <v>29.6947185142194</v>
+        <v>52.0383052814859</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">D8-D7</f>
-        <v>-936.244341265235</v>
+        <v>-894.338363319791</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1593,15 +1602,15 @@
       </c>
       <c r="B10" s="5" t="n">
         <f aca="false">Cozumel!B65</f>
-        <v>76.1578947368421</v>
+        <v>74.8421052631579</v>
       </c>
       <c r="C10" s="5" t="n">
         <f aca="false">Cozumel!C65</f>
-        <v>49.8965517241379</v>
+        <v>49.0344827586207</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">Cozumel!D65</f>
-        <v>37.1025641025641</v>
+        <v>36.4615384615385</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1610,15 +1619,15 @@
       </c>
       <c r="B11" s="4" t="n">
         <f aca="false">Cozumel!B46</f>
-        <v>2118.47591410331</v>
+        <v>2078.35113174695</v>
       </c>
       <c r="C11" s="4" t="n">
         <f aca="false">Cozumel!C46</f>
-        <v>2033.53685432385</v>
+        <v>2022.97446314568</v>
       </c>
       <c r="D11" s="4" t="n">
         <f aca="false">Cozumel!D46</f>
-        <v>2809.47591410331</v>
+        <v>2771.35113174695</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1627,15 +1636,15 @@
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">Cozumel!B23</f>
-        <v>1866.24434126524</v>
+        <v>1822.33836331979</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">Cozumel!C23</f>
-        <v>1891.30528148578</v>
+        <v>1868.96169471851</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">Cozumel!D23</f>
-        <v>2557.24434126524</v>
+        <v>2515.33836331979</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2236,7 +2245,7 @@
         <v>75</v>
       </c>
       <c r="B37" s="9" t="n">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>41</v>
@@ -2250,7 +2259,7 @@
         <v>77</v>
       </c>
       <c r="B38" s="11" t="n">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>73</v>
@@ -2264,32 +2273,32 @@
         <v>79</v>
       </c>
       <c r="B39" s="9" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>31</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B40" s="9" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B41" s="9" t="n">
         <v>530</v>
@@ -2298,40 +2307,40 @@
         <v>41</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B42" s="9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" s="9" t="n">
         <v>85</v>
-      </c>
-      <c r="B43" s="9" t="n">
-        <v>95</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>41</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>31</v>
+        <v>88</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B44" s="9" t="n">
         <v>260</v>
@@ -2340,74 +2349,74 @@
         <v>41</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B45" s="10" t="n">
         <v>5</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B46" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B47" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B48" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B49" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>31</v>
@@ -2415,26 +2424,26 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B50" s="10" t="n">
         <v>10</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B53" s="9" t="n">
         <v>700</v>
@@ -2448,7 +2457,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B54" s="9" t="n">
         <v>1300</v>
@@ -2462,7 +2471,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B55" s="9" t="n">
         <v>1300</v>
@@ -2471,12 +2480,12 @@
         <v>41</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B56" s="9" t="n">
         <v>0</v>
@@ -2485,12 +2494,12 @@
         <v>41</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B57" s="10" t="n">
         <v>6</v>
@@ -2499,228 +2508,228 @@
         <v>65</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B58" s="11" t="n">
         <v>78</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B59" s="11" t="n">
         <v>113</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B60" s="11" t="n">
         <v>358</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B61" s="11" t="n">
         <v>94</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B62" s="11" t="n">
         <v>347</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B63" s="11" t="n">
         <v>69</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B64" s="11" t="n">
         <v>15</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B65" s="11" t="n">
         <v>315</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B66" s="11" t="n">
         <v>67</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B67" s="11" t="n">
         <v>59</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B68" s="11" t="n">
         <v>80</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B69" s="11" t="n">
         <v>22</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B70" s="11" t="n">
         <v>17</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B71" s="11" t="n">
         <v>41</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B72" s="11" t="n">
         <v>45</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B73" s="11" t="n">
         <v>7</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>31</v>
@@ -2728,7 +2737,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B74" s="9" t="n">
         <v>15</v>
@@ -2742,41 +2751,41 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B75" s="10" t="n">
         <v>5</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B76" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B77" s="10" t="n">
         <v>11</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>31</v>
@@ -2784,26 +2793,26 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B78" s="10" t="n">
         <v>22</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B81" s="9" t="n">
         <v>400</v>
@@ -2812,12 +2821,12 @@
         <v>41</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B82" s="9" t="n">
         <v>700</v>
@@ -2826,12 +2835,12 @@
         <v>41</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B83" s="10" t="n">
         <v>4</v>
@@ -2845,7 +2854,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B84" s="10" t="n">
         <v>5</v>
@@ -2859,7 +2868,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B85" s="9" t="n">
         <v>75</v>
@@ -2873,7 +2882,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B86" s="9" t="n">
         <v>50</v>
@@ -2887,7 +2896,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B87" s="9" t="n">
         <v>137</v>
@@ -2896,12 +2905,12 @@
         <v>41</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B88" s="9" t="n">
         <v>140</v>
@@ -2910,54 +2919,54 @@
         <v>41</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B89" s="10" t="n">
         <v>3</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B90" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B91" s="10" t="n">
         <v>1</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B92" s="9" t="n">
         <v>45</v>
@@ -2971,7 +2980,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B93" s="9" t="n">
         <v>70</v>
@@ -2980,26 +2989,26 @@
         <v>41</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B94" s="10" t="n">
         <v>4</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B95" s="9" t="n">
         <v>60</v>
@@ -3013,7 +3022,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B96" s="9" t="n">
         <v>399</v>
@@ -3022,54 +3031,54 @@
         <v>41</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B97" s="8" t="n">
         <v>0.1</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B98" s="10" t="n">
         <v>2</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B99" s="10" t="n">
         <v>3</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B100" s="9" t="n">
         <v>300</v>
@@ -3078,12 +3087,12 @@
         <v>41</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B101" s="9" t="n">
         <v>300</v>
@@ -3092,12 +3101,12 @@
         <v>41</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B102" s="9" t="n">
         <v>240</v>
@@ -3106,12 +3115,12 @@
         <v>41</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B103" s="9" t="n">
         <v>125</v>
@@ -3120,12 +3129,12 @@
         <v>41</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B104" s="9" t="n">
         <v>100</v>
@@ -3139,7 +3148,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B105" s="9" t="n">
         <v>50</v>
@@ -3148,12 +3157,12 @@
         <v>41</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B106" s="9" t="n">
         <v>15</v>
@@ -3167,12 +3176,12 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -3200,22 +3209,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>3</v>
@@ -3229,7 +3238,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$25,Inputs!$B$26)</f>
@@ -3246,7 +3255,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B8" s="4" t="n">
         <f aca="false">2*Inputs!$B$28</f>
@@ -3263,7 +3272,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$29</f>
@@ -3280,7 +3289,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
@@ -3295,7 +3304,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
@@ -3310,7 +3319,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3318,7 +3327,7 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">Inputs!$B$47*Inputs!$B$37</f>
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3327,7 +3336,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>0</v>
@@ -3342,57 +3351,57 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">Inputs!$B$45*Inputs!$B$38/Inputs!$B$7</f>
-        <v>63.8421358096344</v>
+        <v>69.9361578641904</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">(Inputs!$B$49+Inputs!$B$47)*Inputs!$B$38/Inputs!$B$7</f>
-        <v>38.3052814857806</v>
+        <v>41.9616947185142</v>
       </c>
       <c r="D14" s="4" t="n">
         <f aca="false">Inputs!$B$45*Inputs!$B$38/Inputs!$B$7</f>
-        <v>63.8421358096344</v>
+        <v>69.9361578641904</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">Inputs!$B$45*Inputs!$B$39</f>
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="C15" s="4" t="n">
         <f aca="false">Inputs!$B$47*Inputs!$B$39</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D15" s="4" t="n">
         <f aca="false">Inputs!$B$45*Inputs!$B$39</f>
-        <v>125</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">Inputs!$B$40</f>
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="4" t="n">
         <f aca="false">Inputs!$B$40</f>
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B17" s="4" t="n">
         <v>0</v>
@@ -3402,12 +3411,12 @@
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">6*Inputs!$B$42</f>
-        <v>66</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B18" s="4" t="n">
         <v>0</v>
@@ -3417,12 +3426,12 @@
       </c>
       <c r="D18" s="4" t="n">
         <f aca="false">Inputs!$B$43</f>
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">Inputs!$B$32*Inputs!$B$21</f>
@@ -3439,7 +3448,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B20" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -3456,7 +3465,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B21" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -3473,41 +3482,41 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">SUM(B7:B21)</f>
-        <v>2245.24434126524</v>
+        <v>2201.33836331979</v>
       </c>
       <c r="C22" s="12" t="n">
         <f aca="false">SUM(C7:C21)</f>
-        <v>2270.30528148578</v>
+        <v>2247.96169471851</v>
       </c>
       <c r="D22" s="12" t="n">
         <f aca="false">SUM(D7:D21)</f>
-        <v>2936.24434126524</v>
+        <v>2894.33836331979</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B23" s="4" t="n">
         <f aca="false">B22-SUM(B19:B21)</f>
-        <v>1866.24434126524</v>
+        <v>1822.33836331979</v>
       </c>
       <c r="C23" s="4" t="n">
         <f aca="false">C22-SUM(C19:C21)</f>
-        <v>1891.30528148578</v>
+        <v>1868.96169471851</v>
       </c>
       <c r="D23" s="4" t="n">
         <f aca="false">D22-SUM(D19:D21)</f>
-        <v>2557.24434126524</v>
+        <v>2515.33836331979</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B24" s="4" t="n">
         <f aca="false">Inputs!$B$15</f>
@@ -3524,24 +3533,24 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B25" s="4" t="n">
         <f aca="false">B24-B22</f>
-        <v>-245.244341265235</v>
+        <v>-201.338363319791</v>
       </c>
       <c r="C25" s="4" t="n">
         <f aca="false">C24-C22</f>
-        <v>29.6947185142194</v>
+        <v>52.0383052814859</v>
       </c>
       <c r="D25" s="4" t="n">
         <f aca="false">D24-D22</f>
-        <v>-936.244341265235</v>
+        <v>-894.338363319791</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B26" s="4" t="n">
         <f aca="false">Inputs!$B$44</f>
@@ -3558,12 +3567,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>3</v>
@@ -3577,7 +3586,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B31" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$25,Inputs!$B$26)</f>
@@ -3594,7 +3603,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B32" s="4" t="n">
         <f aca="false">2*Inputs!$B$28</f>
@@ -3611,7 +3620,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B33" s="4" t="n">
         <f aca="false">Inputs!$B$33*Inputs!$B$29</f>
@@ -3628,7 +3637,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B34" s="4" t="n">
         <v>0</v>
@@ -3643,7 +3652,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>0</v>
@@ -3658,7 +3667,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3666,7 +3675,7 @@
       </c>
       <c r="C36" s="4" t="n">
         <f aca="false">Inputs!$B$48*Inputs!$B$37</f>
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D36" s="4" t="n">
         <f aca="false">Inputs!$B$36/Inputs!$B$7</f>
@@ -3675,7 +3684,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B37" s="4" t="n">
         <v>0</v>
@@ -3690,57 +3699,57 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">Inputs!$B$46*Inputs!$B$38/Inputs!$B$7</f>
-        <v>51.0737086477075</v>
+        <v>55.9489262913523</v>
       </c>
       <c r="C38" s="4" t="n">
         <f aca="false">(Inputs!$B$49+Inputs!$B$48)*Inputs!$B$38/Inputs!$B$7</f>
-        <v>25.5368543238537</v>
+        <v>27.9744631456761</v>
       </c>
       <c r="D38" s="4" t="n">
         <f aca="false">Inputs!$B$46*Inputs!$B$38/Inputs!$B$7</f>
-        <v>51.0737086477075</v>
+        <v>55.9489262913523</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">Inputs!$B$46*Inputs!$B$39</f>
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C39" s="4" t="n">
         <f aca="false">Inputs!$B$48*Inputs!$B$39</f>
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D39" s="4" t="n">
         <f aca="false">Inputs!$B$46*Inputs!$B$39</f>
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B40" s="4" t="n">
         <f aca="false">Inputs!$B$40</f>
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="C40" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D40" s="4" t="n">
         <f aca="false">Inputs!$B$40</f>
-        <v>30</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B41" s="4" t="n">
         <v>0</v>
@@ -3750,12 +3759,12 @@
       </c>
       <c r="D41" s="4" t="n">
         <f aca="false">6*Inputs!$B$42</f>
-        <v>66</v>
+        <v>78</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>0</v>
@@ -3765,12 +3774,12 @@
       </c>
       <c r="D42" s="4" t="n">
         <f aca="false">Inputs!$B$43</f>
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B43" s="4" t="n">
         <f aca="false">Inputs!$B$33*Inputs!$B$21</f>
@@ -3787,7 +3796,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B44" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -3804,7 +3813,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -3821,41 +3830,41 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B46" s="12" t="n">
         <f aca="false">SUM(B31:B45)</f>
-        <v>2118.47591410331</v>
+        <v>2078.35113174695</v>
       </c>
       <c r="C46" s="12" t="n">
         <f aca="false">SUM(C31:C45)</f>
-        <v>2033.53685432385</v>
+        <v>2022.97446314568</v>
       </c>
       <c r="D46" s="12" t="n">
         <f aca="false">SUM(D31:D45)</f>
-        <v>2809.47591410331</v>
+        <v>2771.35113174695</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B47" s="4" t="n">
         <f aca="false">B46-SUM(B43:B45)</f>
-        <v>1774.47591410331</v>
+        <v>1734.35113174695</v>
       </c>
       <c r="C47" s="4" t="n">
         <f aca="false">C46-SUM(C43:C45)</f>
-        <v>1689.53685432385</v>
+        <v>1678.97446314568</v>
       </c>
       <c r="D47" s="4" t="n">
         <f aca="false">D46-SUM(D43:D45)</f>
-        <v>2465.47591410331</v>
+        <v>2427.35113174695</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B48" s="4" t="n">
         <f aca="false">Inputs!$B$15</f>
@@ -3872,41 +3881,41 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B49" s="4" t="n">
         <f aca="false">B48-B46</f>
-        <v>-118.475914103308</v>
+        <v>-78.3511317469529</v>
       </c>
       <c r="C49" s="4" t="n">
         <f aca="false">C48-C46</f>
-        <v>266.463145676146</v>
+        <v>277.025536854324</v>
       </c>
       <c r="D49" s="4" t="n">
         <f aca="false">D48-D46</f>
-        <v>-809.475914103308</v>
+        <v>-771.351131746953</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2"/>
       <c r="B53" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B54" s="10" t="n">
         <v>20</v>
@@ -3920,7 +3929,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B55" s="2" t="n">
         <f aca="false">B54-1</f>
@@ -3937,7 +3946,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B56" s="2" t="n">
         <f aca="false">INT(B55/Inputs!$B$50)</f>
@@ -3954,80 +3963,80 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B57" s="4" t="n">
         <f aca="false">B12+B14+B15</f>
-        <v>798.244341265235</v>
+        <v>779.338363319791</v>
       </c>
       <c r="C57" s="4" t="n">
         <f aca="false">B12+B14+B15</f>
-        <v>798.244341265235</v>
+        <v>779.338363319791</v>
       </c>
       <c r="D57" s="4" t="n">
         <f aca="false">B12+B14+B15</f>
-        <v>798.244341265235</v>
+        <v>779.338363319791</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B58" s="4" t="n">
         <f aca="false">B22</f>
-        <v>2245.24434126524</v>
+        <v>2201.33836331979</v>
       </c>
       <c r="C58" s="4" t="n">
         <f aca="false">B22</f>
-        <v>2245.24434126524</v>
+        <v>2201.33836331979</v>
       </c>
       <c r="D58" s="4" t="n">
         <f aca="false">B22</f>
-        <v>2245.24434126524</v>
+        <v>2201.33836331979</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B59" s="4" t="n">
         <f aca="false">MIN(B56,1)*B57</f>
-        <v>798.244341265235</v>
+        <v>779.338363319791</v>
       </c>
       <c r="C59" s="4" t="n">
         <f aca="false">MIN(C56,1)*C57</f>
-        <v>798.244341265235</v>
+        <v>779.338363319791</v>
       </c>
       <c r="D59" s="4" t="n">
         <f aca="false">MIN(D56,1)*D57</f>
-        <v>798.244341265235</v>
+        <v>779.338363319791</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B62" s="4" t="n">
         <f aca="false">B58-B59</f>
-        <v>1447</v>
+        <v>1422</v>
       </c>
       <c r="C62" s="4" t="n">
         <f aca="false">C58-C59</f>
-        <v>1447</v>
+        <v>1422</v>
       </c>
       <c r="D62" s="4" t="n">
         <f aca="false">D58-D59</f>
-        <v>1447</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B63" s="4" t="n">
         <v>0</v>
@@ -4041,119 +4050,119 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B65" s="5" t="n">
         <f aca="false">(B58-B59)/B55</f>
-        <v>76.1578947368421</v>
+        <v>74.8421052631579</v>
       </c>
       <c r="C65" s="5" t="n">
         <f aca="false">(C58-C59)/C55</f>
-        <v>49.8965517241379</v>
+        <v>49.0344827586207</v>
       </c>
       <c r="D65" s="5" t="n">
         <f aca="false">(D58-D59)/D55</f>
-        <v>37.1025641025641</v>
+        <v>36.4615384615385</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B66" s="4" t="n">
         <f aca="false">B22+B65</f>
-        <v>2321.40223600208</v>
+        <v>2276.18046858295</v>
       </c>
       <c r="C66" s="4" t="n">
         <f aca="false">B22+C65</f>
-        <v>2295.14089298937</v>
+        <v>2250.37284607841</v>
       </c>
       <c r="D66" s="4" t="n">
         <f aca="false">B22+D65</f>
-        <v>2282.3469053678</v>
+        <v>2237.79990178133</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B67" s="4" t="n">
         <f aca="false">C22+B65</f>
-        <v>2346.46317622262</v>
+        <v>2322.80379998167</v>
       </c>
       <c r="C67" s="4" t="n">
         <f aca="false">C22+C65</f>
-        <v>2320.20183320992</v>
+        <v>2296.99617747713</v>
       </c>
       <c r="D67" s="4" t="n">
         <f aca="false">C22+D65</f>
-        <v>2307.40784558834</v>
+        <v>2284.42323318005</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B69" s="5" t="n">
         <f aca="false">B58/B55</f>
-        <v>118.170754803433</v>
+        <v>115.859913858936</v>
       </c>
       <c r="C69" s="5" t="n">
         <f aca="false">B58/C55</f>
-        <v>77.4222186643185</v>
+        <v>75.9082194248204</v>
       </c>
       <c r="D69" s="5" t="n">
         <f aca="false">B58/D55</f>
-        <v>57.5703677247496</v>
+        <v>56.4445734184562</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B70" s="4" t="n">
         <f aca="false">B22+B69</f>
-        <v>2363.41509606867</v>
+        <v>2317.19827717873</v>
       </c>
       <c r="C70" s="4" t="n">
         <f aca="false">B22+C69</f>
-        <v>2322.66655992955</v>
+        <v>2277.24658274461</v>
       </c>
       <c r="D70" s="4" t="n">
         <f aca="false">B22+D69</f>
-        <v>2302.81470898999</v>
+        <v>2257.78293673825</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B71" s="4" t="n">
         <f aca="false">C22+B69</f>
-        <v>2388.47603628921</v>
+        <v>2363.82160857745</v>
       </c>
       <c r="C71" s="4" t="n">
         <f aca="false">C22+C69</f>
-        <v>2347.7275001501</v>
+        <v>2323.86991414333</v>
       </c>
       <c r="D71" s="4" t="n">
         <f aca="false">C22+D69</f>
-        <v>2327.87564921053</v>
+        <v>2304.40626813697</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B72" s="2" t="n">
         <f aca="false">MAX(B56-1,0)</f>
@@ -4170,26 +4179,26 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B77" s="4" t="n">
         <f aca="false">Inputs!$B$25</f>
@@ -4206,64 +4215,64 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B78" s="4" t="n">
         <f aca="false">B22-B7+B77</f>
-        <v>2129.24434126524</v>
+        <v>2085.33836331979</v>
       </c>
       <c r="C78" s="4" t="n">
         <f aca="false">B22-B7+C77</f>
-        <v>2245.24434126524</v>
+        <v>2201.33836331979</v>
       </c>
       <c r="D78" s="4" t="n">
         <f aca="false">B22-B7+D77</f>
-        <v>2361.24434126524</v>
+        <v>2317.33836331979</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">C22-B7+B77</f>
-        <v>2154.30528148578</v>
+        <v>2131.96169471851</v>
       </c>
       <c r="C79" s="4" t="n">
         <f aca="false">C22-B7+C77</f>
-        <v>2270.30528148578</v>
+        <v>2247.96169471851</v>
       </c>
       <c r="D79" s="4" t="n">
         <f aca="false">C22-B7+D77</f>
-        <v>2386.30528148578</v>
+        <v>2363.96169471851</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B22-B7+Inputs!$B$27</f>
-        <v>1961.24434126524</v>
+        <v>1917.33836331979</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B83" s="13" t="n">
         <f aca="false">Inputs!$B$7*0.9</f>
@@ -4280,74 +4289,74 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B84" s="14" t="n">
         <f aca="false">Inputs!$B$36+Inputs!$B$45*Inputs!$B$38</f>
-        <v>11600</v>
+        <v>11705</v>
       </c>
       <c r="C84" s="14" t="n">
         <f aca="false">Inputs!$B$36+Inputs!$B$45*Inputs!$B$38</f>
-        <v>11600</v>
+        <v>11705</v>
       </c>
       <c r="D84" s="14" t="n">
         <f aca="false">Inputs!$B$36+Inputs!$B$45*Inputs!$B$38</f>
-        <v>11600</v>
+        <v>11705</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B85" s="4" t="n">
         <f aca="false">B22-B12-B14+B84/B83</f>
-        <v>2320.04926807248</v>
+        <v>2276.82040368866</v>
       </c>
       <c r="C85" s="4" t="n">
         <f aca="false">B22-B12-B14+C84/C83</f>
-        <v>2245.24434126524</v>
+        <v>2201.33836331979</v>
       </c>
       <c r="D85" s="4" t="n">
         <f aca="false">B22-B12-B14+D84/D83</f>
-        <v>2184.04031024112</v>
+        <v>2139.58033029072</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B91" s="4" t="n">
         <f aca="false">B58-B57</f>
-        <v>1447</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">Inputs!$B$15-B22</f>
-        <v>-245.244341265235</v>
+        <v>-201.338363319791</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B93" s="2" t="str">
         <f aca="false">IF(B92&gt;0,ROUNDUP(B91/B92,0)+1,"not viable at this price")</f>
@@ -4356,153 +4365,153 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B94" s="4" t="n">
         <f aca="false">Inputs!$B$16-C22</f>
-        <v>29.6947185142194</v>
+        <v>52.0383052814859</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B95" s="2" t="n">
         <f aca="false">IF(B94&gt;0,ROUNDUP(B91/B94,0)+1,"not viable at this price")</f>
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C101" s="4" t="n">
         <v>600</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C102" s="4" t="n">
         <f aca="false">0.25*B12</f>
         <v>152.3505513639</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C103" s="4" t="n">
         <f aca="false">Inputs!$B$29</f>
         <v>54</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C105" s="4" t="n">
         <f aca="false">B22-600</f>
-        <v>1645.24434126524</v>
+        <v>1601.33836331979</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C106" s="2"/>
       <c r="D106" s="2" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="C107" s="2"/>
       <c r="D107" s="2" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="C108" s="2"/>
       <c r="D108" s="2" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -4530,22 +4539,22 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>3</v>
@@ -4559,7 +4568,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B7" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$53,Inputs!$B$54)</f>
@@ -4576,7 +4585,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B8" s="4" t="n">
         <f aca="false">2*Inputs!$B$71*Inputs!$B$6</f>
@@ -4593,7 +4602,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$58*Inputs!$B$6</f>
@@ -4610,7 +4619,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B10" s="4" t="n">
         <v>0</v>
@@ -4625,7 +4634,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B11" s="4" t="n">
         <v>0</v>
@@ -4640,7 +4649,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">Inputs!$B$62*Inputs!$B$6</f>
@@ -4657,7 +4666,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B13" s="4" t="n">
         <v>0</v>
@@ -4672,7 +4681,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
@@ -4689,7 +4698,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">(Inputs!$B$66+Inputs!$B$67)*Inputs!$B$6</f>
@@ -4706,7 +4715,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">Inputs!$B$72*Inputs!$B$6</f>
@@ -4723,7 +4732,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">Inputs!$B$73*Inputs!$B$6</f>
@@ -4740,7 +4749,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B18" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
@@ -4757,7 +4766,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -4774,7 +4783,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B20" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -4791,7 +4800,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">SUM(B7:B20)</f>
@@ -4808,7 +4817,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B22" s="4" t="n">
         <f aca="false">B21-SUM(B18:B20)</f>
@@ -4825,7 +4834,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B23" s="4" t="n">
         <f aca="false">Inputs!$B$17</f>
@@ -4842,7 +4851,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B24" s="4" t="n">
         <f aca="false">B23-B21</f>
@@ -4859,12 +4868,12 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>3</v>
@@ -4878,7 +4887,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$53,Inputs!$B$54)</f>
@@ -4895,7 +4904,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B30" s="4" t="n">
         <f aca="false">2*Inputs!$B$69*Inputs!$B$6</f>
@@ -4912,7 +4921,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B31" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$59*Inputs!$B$6</f>
@@ -4929,7 +4938,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>0</v>
@@ -4944,7 +4953,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B33" s="4" t="n">
         <v>0</v>
@@ -4959,7 +4968,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B34" s="4" t="n">
         <f aca="false">Inputs!$B$62*Inputs!$B$6</f>
@@ -4976,7 +4985,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B35" s="4" t="n">
         <v>0</v>
@@ -4991,7 +5000,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
@@ -5008,7 +5017,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B37" s="4" t="n">
         <f aca="false">(Inputs!$B$66+Inputs!$B$67)*Inputs!$B$6</f>
@@ -5025,7 +5034,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">Inputs!$B$72*Inputs!$B$6</f>
@@ -5042,7 +5051,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">Inputs!$B$73*Inputs!$B$6</f>
@@ -5059,7 +5068,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B40" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
@@ -5076,7 +5085,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B41" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -5093,7 +5102,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B42" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -5110,7 +5119,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B43" s="12" t="n">
         <f aca="false">SUM(B29:B42)</f>
@@ -5127,7 +5136,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B44" s="4" t="n">
         <f aca="false">B43-SUM(B40:B42)</f>
@@ -5144,7 +5153,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Inputs!$B$17</f>
@@ -5161,7 +5170,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B46" s="4" t="n">
         <f aca="false">B45-B43</f>
@@ -5178,7 +5187,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B47" s="4" t="n">
         <f aca="false">Inputs!$B$56</f>
@@ -5195,24 +5204,24 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2"/>
       <c r="B51" s="3" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B52" s="10" t="n">
         <v>15</v>
@@ -5226,7 +5235,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B53" s="2" t="n">
         <f aca="false">B52-1</f>
@@ -5243,7 +5252,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B54" s="2" t="n">
         <f aca="false">IF(B52&gt;=Inputs!$B$78,2,IF(B52&gt;=Inputs!$B$77,1,0))</f>
@@ -5260,7 +5269,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B55" s="4" t="n">
         <f aca="false">B9+B8+B12</f>
@@ -5277,7 +5286,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B56" s="4" t="n">
         <f aca="false">B21</f>
@@ -5294,7 +5303,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B57" s="4" t="n">
         <f aca="false">MIN(B54,1)*B55</f>
@@ -5311,12 +5320,12 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B60" s="4" t="n">
         <f aca="false">B56-B57</f>
@@ -5333,7 +5342,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B61" s="4" t="n">
         <v>0</v>
@@ -5347,12 +5356,12 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B63" s="5" t="n">
         <f aca="false">(B56-B57)/B53</f>
@@ -5369,7 +5378,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B64" s="4" t="n">
         <f aca="false">B21+B63</f>
@@ -5386,7 +5395,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B65" s="4" t="n">
         <f aca="false">C21+B63</f>
@@ -5403,12 +5412,12 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B67" s="5" t="n">
         <f aca="false">B56/B53</f>
@@ -5425,7 +5434,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B68" s="4" t="n">
         <f aca="false">B21+B67</f>
@@ -5442,7 +5451,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B69" s="4" t="n">
         <f aca="false">C21+B67</f>
@@ -5459,7 +5468,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B70" s="4" t="n">
         <v>0</v>
@@ -5474,7 +5483,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B71" s="4" t="n">
         <v>0</v>
@@ -5489,26 +5498,26 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B76" s="4" t="n">
         <f aca="false">Inputs!$B$53</f>
@@ -5525,7 +5534,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B77" s="4" t="n">
         <f aca="false">B21-B7+B76</f>
@@ -5542,7 +5551,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B78" s="4" t="n">
         <f aca="false">C21-B7+B76</f>
@@ -5559,7 +5568,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">D21-B7+B76</f>
@@ -5576,7 +5585,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B21-B7+Inputs!$B$55-B8+2*Inputs!$B$69*Inputs!$B$6</f>
@@ -5585,21 +5594,21 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B83" s="15" t="n">
         <f aca="false">Inputs!$B$6*0.9</f>
@@ -5616,7 +5625,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B84" s="4" t="n">
         <f aca="false">(B7+B18+B19+B20)+(B21-(B7+B18+B19+B20))*B83/Inputs!$B$6</f>
@@ -5633,7 +5642,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="2" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B85" s="4" t="n">
         <f aca="false">(C7+C18+C19+C20)+(C21-(C7+C18+C19+C20))*B83/Inputs!$B$6</f>
@@ -5650,12 +5659,12 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B89" s="4" t="n">
         <f aca="false">B56-B55</f>
@@ -5664,7 +5673,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B90" s="4" t="n">
         <f aca="false">Inputs!$B$17-B21</f>
@@ -5673,7 +5682,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B91" s="2" t="n">
         <f aca="false">IF(B90&gt;0,ROUNDUP(B89/B90,0)+1,"not viable at this price")</f>
@@ -5682,7 +5691,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">Inputs!$B$17-C21</f>
@@ -5691,7 +5700,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B93" s="2" t="str">
         <f aca="false">IF(B92&gt;0,ROUNDUP(B89/B92,0)+1,"not viable at this price")</f>
@@ -5700,106 +5709,106 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="2" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C99" s="4" t="n">
         <v>700</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="2" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C100" s="4" t="n">
         <f aca="false">0.5*(B9+B8+B12)</f>
         <v>514.20525</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="2" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C102" s="4" t="n">
         <f aca="false">B21-700</f>
         <v>1877.475</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="C103" s="2"/>
       <c r="D103" s="2" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
       <c r="D104" s="2" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -5827,17 +5836,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>8</v>
@@ -5851,26 +5860,26 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$81,Inputs!$B$82)</f>
@@ -5887,7 +5896,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B10" s="4" t="n">
         <f aca="false">(ROUNDUP(B5/Inputs!$B$94,0)*(Inputs!$B$83*Inputs!$B$93+Inputs!$B$95))/B5</f>
@@ -5904,7 +5913,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B11" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$85</f>
@@ -5921,7 +5930,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B12" s="4" t="n">
         <f aca="false">(Inputs!$B$89-Inputs!$B$91)*Inputs!$B$87</f>
@@ -5938,7 +5947,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B13" s="4" t="n">
         <f aca="false">Inputs!$B$91*Inputs!$B$88</f>
@@ -5955,7 +5964,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">Inputs!$B$92</f>
@@ -5972,7 +5981,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B15" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$21</f>
@@ -5989,7 +5998,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6006,7 +6015,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6023,7 +6032,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">SUM(B9:B17)</f>
@@ -6040,7 +6049,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">B18-SUM(B15:B17)</f>
@@ -6057,7 +6066,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B20" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6074,7 +6083,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B21" s="4" t="n">
         <f aca="false">B20-B18</f>
@@ -6091,26 +6100,26 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B26" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$81,Inputs!$B$82)</f>
@@ -6127,7 +6136,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">(ROUNDUP(B5/Inputs!$B$94,0)*(Inputs!$B$84*Inputs!$B$93+Inputs!$B$95))/B5</f>
@@ -6144,7 +6153,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$85</f>
@@ -6161,7 +6170,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">(Inputs!$B$90-Inputs!$B$91)*Inputs!$B$87</f>
@@ -6178,7 +6187,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B30" s="4" t="n">
         <f aca="false">Inputs!$B$91*Inputs!$B$88</f>
@@ -6195,7 +6204,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B31" s="4" t="n">
         <f aca="false">Inputs!$B$92</f>
@@ -6212,7 +6221,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B32" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$21</f>
@@ -6229,7 +6238,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B33" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6246,7 +6255,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B34" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6263,7 +6272,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B35" s="12" t="n">
         <f aca="false">SUM(B26:B34)</f>
@@ -6280,7 +6289,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">B35-SUM(B32:B34)</f>
@@ -6297,7 +6306,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B37" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6314,7 +6323,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B38" s="4" t="n">
         <f aca="false">B37-B35</f>
@@ -6331,26 +6340,26 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B43" s="4" t="n">
         <f aca="false">Inputs!$B$100+Inputs!$B$101</f>
@@ -6367,7 +6376,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B44" s="4" t="n">
         <f aca="false">Inputs!$B$105</f>
@@ -6384,7 +6393,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B45" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$103</f>
@@ -6401,7 +6410,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B46" s="4" t="n">
         <f aca="false">Inputs!$B$98*Inputs!$B$96*(1+Inputs!$B$97)</f>
@@ -6418,7 +6427,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B47" s="4" t="n">
         <f aca="false">Inputs!$B$98*Inputs!$B$106</f>
@@ -6435,7 +6444,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B48" s="4" t="n">
         <f aca="false">Inputs!$B$83*Inputs!$B$21</f>
@@ -6452,7 +6461,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B49" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6469,7 +6478,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B50" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6486,7 +6495,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B51" s="12" t="n">
         <f aca="false">SUM(B43:B50)</f>
@@ -6503,7 +6512,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B52" s="4" t="n">
         <f aca="false">B51-SUM(B48:B50)</f>
@@ -6520,7 +6529,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B53" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6537,7 +6546,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B54" s="4" t="n">
         <f aca="false">B53-B51</f>
@@ -6554,7 +6563,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B55" s="12" t="n">
         <f aca="false">B51-B18</f>
@@ -6571,7 +6580,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B56" s="4" t="n">
         <f aca="false">Inputs!$B$101-Inputs!$B$102</f>
@@ -6588,26 +6597,26 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B61" s="4" t="n">
         <f aca="false">Inputs!$B$100+Inputs!$B$101</f>
@@ -6624,7 +6633,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B62" s="4" t="n">
         <f aca="false">Inputs!$B$105</f>
@@ -6641,7 +6650,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B63" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$103</f>
@@ -6658,7 +6667,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B64" s="4" t="n">
         <f aca="false">Inputs!$B$99*Inputs!$B$96*(1+Inputs!$B$97)</f>
@@ -6675,7 +6684,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B65" s="4" t="n">
         <f aca="false">Inputs!$B$99*Inputs!$B$106</f>
@@ -6692,7 +6701,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B66" s="4" t="n">
         <f aca="false">Inputs!$B$84*Inputs!$B$21</f>
@@ -6709,7 +6718,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B67" s="4" t="n">
         <f aca="false">Inputs!$B$22</f>
@@ -6726,7 +6735,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B68" s="4" t="n">
         <f aca="false">Inputs!$B$20</f>
@@ -6743,7 +6752,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B69" s="12" t="n">
         <f aca="false">SUM(B61:B68)</f>
@@ -6760,7 +6769,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B70" s="4" t="n">
         <f aca="false">B69-SUM(B66:B68)</f>
@@ -6777,7 +6786,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B71" s="4" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -6794,7 +6803,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B72" s="4" t="n">
         <f aca="false">B71-B69</f>
@@ -6811,7 +6820,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B73" s="12" t="n">
         <f aca="false">B69-B35</f>
@@ -6828,17 +6837,17 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B78" s="2" t="n">
         <f aca="false">B5-1</f>
@@ -6855,7 +6864,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">B12+B13</f>
@@ -6872,7 +6881,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B18</f>
@@ -6889,7 +6898,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B81" s="4" t="n">
         <f aca="false">B80-B79</f>
@@ -6906,7 +6915,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B82" s="5" t="n">
         <f aca="false">(B80-B79)/B78</f>
@@ -6923,7 +6932,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B83" s="5" t="n">
         <f aca="false">B80/B78</f>
@@ -6940,7 +6949,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B84" s="4" t="n">
         <f aca="false">B18+B83</f>
@@ -6957,26 +6966,26 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B89" s="4" t="n">
         <f aca="false">Inputs!$B$81</f>
@@ -6993,7 +7002,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="2" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B90" s="4" t="n">
         <f aca="false">C18-C9+B89</f>
@@ -7010,7 +7019,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="2" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B91" s="4" t="n">
         <f aca="false">C18-C13+Inputs!$B$87</f>
@@ -7019,7 +7028,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="2" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">C18-Inputs!$B$83*(Inputs!$B$85-Inputs!$B$86)</f>
@@ -7028,12 +7037,12 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="2" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B96" s="4" t="n">
         <f aca="false">Inputs!$B$14-C18</f>
@@ -7042,7 +7051,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="2" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B97" s="2" t="str">
         <f aca="false">IF(B96&gt;0,ROUNDUP(C80/B96,0)+1,"not viable at this price")</f>
@@ -7051,120 +7060,120 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="2" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="2" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C104" s="4" t="n">
         <v>400</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="2" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="C105" s="4" t="n">
         <f aca="false">AVERAGE(Inputs!$B$81,Inputs!$B$82)</f>
         <v>550</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="2" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C106" s="4" t="n">
         <f aca="false">Inputs!$B$85</f>
         <v>75</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="2" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="C107" s="4" t="n">
         <f aca="false">0.25*(C12+C13)</f>
         <v>103.5</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C108" s="4" t="n">
         <f aca="false">C18-400</f>
         <v>1320</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="2" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C109" s="4" t="n">
         <f aca="false">Inputs!$B$98*Inputs!$B$96*(1+Inputs!$B$97)</f>
         <v>877.8</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
All three trips confirmed go; Egypt shortened to Sat 2 – Fri 8 Jan; off activities planned in-house; routine procedure rewritten
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/december_pricing.xlsx
+++ b/december-plan/pricing/december_pricing.xlsx
@@ -62,7 +62,7 @@
     <t xml:space="preserve">Core only (excl. meals, tips, insurance), 6 nights</t>
   </si>
   <si>
-    <t xml:space="preserve">Egypt, Marsa Shagra (Sat 2 – Sat 9 Jan)</t>
+    <t xml:space="preserve">Egypt, Marsa Shagra (Sat 2 – Fri 8 Jan)</t>
   </si>
   <si>
     <t xml:space="preserve">All-in per person, Royal Tent, via Hurghada</t>
@@ -332,7 +332,7 @@
     <t xml:space="preserve">QUOTED 2026-09-22: Aldora 1 comp at 10+ paid; Sand Dollar one free diver</t>
   </si>
   <si>
-    <t xml:space="preserve">Egypt (Marsa Shagra), Sat 2 – Sat 9 Jan 2027, 6 nights on the ground</t>
+    <t xml:space="preserve">Egypt (Marsa Shagra), Sat 2 – Fri 8 Jan 2027, 6 nights on the ground</t>
   </si>
   <si>
     <t xml:space="preserve">Flight PHL–HRG return via Lufthansa Group hub, low</t>
@@ -353,7 +353,7 @@
     <t xml:space="preserve">QUOTE NEEDED; one-way ~USD 550 seen</t>
   </si>
   <si>
-    <t xml:space="preserve">Nights on the ground (Sun 3 – Sat 9)</t>
+    <t xml:space="preserve">Nights on the ground (Sun 3 – Fri 8; shortened 23 Sep)</t>
   </si>
   <si>
     <t xml:space="preserve">Royal Tent, full board, pp/night sharing</t>
@@ -428,10 +428,10 @@
     <t xml:space="preserve">Incidentals per day on full board</t>
   </si>
   <si>
-    <t xml:space="preserve">Certified dive days (Mon–Fri, Fri morning only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beginner dive days after course (Thu–Fri)</t>
+    <t xml:space="preserve">Certified dive days (Mon–Thu, Thu morning only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beginner dive days after course (Thu morning)</t>
   </si>
   <si>
     <t xml:space="preserve">RSDS free places: threshold for first free guest</t>
@@ -854,7 +854,7 @@
     <t xml:space="preserve">Per policy snippets</t>
   </si>
   <si>
-    <t xml:space="preserve">Egypt, Marsa Shagra — Sat 2 – Sat 9 Jan 2027 (6 nights on the ground)</t>
+    <t xml:space="preserve">Egypt, Marsa Shagra — Sat 2 – Fri 8 Jan 2027 (6 nights on the ground)</t>
   </si>
   <si>
     <t xml:space="preserve">All figures per person, USD, converted from EUR at the Inputs rate. Full board included in lodging. Flights PHL–HRG via a Lufthansa Group hub at the band midpoint; transfers from Hurghada (3 h) unless RMF proves bookable.</t>
@@ -1670,15 +1670,15 @@
       </c>
       <c r="B16" s="4" t="n">
         <f aca="false">January!B21</f>
-        <v>2577.475</v>
+        <v>2455.8505</v>
       </c>
       <c r="C16" s="4" t="n">
         <f aca="false">January!C21</f>
-        <v>2727.6665</v>
+        <v>2526.9335</v>
       </c>
       <c r="D16" s="4" t="n">
         <f aca="false">January!D21</f>
-        <v>2962.699</v>
+        <v>2841.0745</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1687,15 +1687,15 @@
       </c>
       <c r="B17" s="4" t="n">
         <f aca="false">January!B43</f>
-        <v>2774.673</v>
+        <v>2612.921</v>
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">January!C43</f>
-        <v>2924.8645</v>
+        <v>2684.004</v>
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">January!D43</f>
-        <v>3159.897</v>
+        <v>2998.145</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1721,15 +1721,15 @@
       </c>
       <c r="B19" s="4" t="n">
         <f aca="false">B18-B16</f>
-        <v>122.525</v>
+        <v>244.1495</v>
       </c>
       <c r="C19" s="4" t="n">
         <f aca="false">C18-C16</f>
-        <v>-27.6665000000003</v>
+        <v>173.0665</v>
       </c>
       <c r="D19" s="4" t="n">
         <f aca="false">D18-D16</f>
-        <v>-262.699</v>
+        <v>-141.0745</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1738,15 +1738,15 @@
       </c>
       <c r="B20" s="5" t="n">
         <f aca="false">January!B63</f>
-        <v>110.647464285714</v>
+        <v>108.347642857143</v>
       </c>
       <c r="C20" s="5" t="n">
         <f aca="false">January!C63</f>
-        <v>81.5297105263158</v>
+        <v>79.8351052631579</v>
       </c>
       <c r="D20" s="5" t="n">
         <f aca="false">January!D63</f>
-        <v>64.5443541666667</v>
+        <v>63.2027916666667</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1755,15 +1755,15 @@
       </c>
       <c r="B21" s="4" t="n">
         <f aca="false">January!B22</f>
-        <v>2318.475</v>
+        <v>2211.8505</v>
       </c>
       <c r="C21" s="4" t="n">
         <f aca="false">January!C22</f>
-        <v>2468.6665</v>
+        <v>2282.9335</v>
       </c>
       <c r="D21" s="4" t="n">
         <f aca="false">January!D22</f>
-        <v>2703.699</v>
+        <v>2597.0745</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2502,7 +2502,7 @@
         <v>109</v>
       </c>
       <c r="B57" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>65</v>
@@ -2754,7 +2754,7 @@
         <v>134</v>
       </c>
       <c r="B75" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>92</v>
@@ -2768,7 +2768,7 @@
         <v>135</v>
       </c>
       <c r="B76" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>92</v>
@@ -4606,15 +4606,15 @@
       </c>
       <c r="B9" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$58*Inputs!$B$6</f>
-        <v>536.562</v>
+        <v>447.135</v>
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$58*Inputs!$B$6</f>
-        <v>536.562</v>
+        <v>447.135</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$58*Inputs!$B$6</f>
-        <v>536.562</v>
+        <v>447.135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4657,7 +4657,7 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">Inputs!$B$76*Inputs!$B$63*Inputs!$B$6</f>
-        <v>158.217</v>
+        <v>79.1085</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">Inputs!$B$62*Inputs!$B$6</f>
@@ -4685,15 +4685,15 @@
       </c>
       <c r="B14" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
-        <v>85.9875</v>
+        <v>68.79</v>
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Inputs!$B$76*Inputs!$B$64*Inputs!$B$6</f>
-        <v>34.395</v>
+        <v>17.1975</v>
       </c>
       <c r="D14" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
-        <v>85.9875</v>
+        <v>68.79</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4753,15 +4753,15 @@
       </c>
       <c r="B18" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C18" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D18" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4804,15 +4804,15 @@
       </c>
       <c r="B21" s="12" t="n">
         <f aca="false">SUM(B7:B20)</f>
-        <v>2577.475</v>
+        <v>2455.8505</v>
       </c>
       <c r="C21" s="12" t="n">
         <f aca="false">SUM(C7:C20)</f>
-        <v>2727.6665</v>
+        <v>2526.9335</v>
       </c>
       <c r="D21" s="12" t="n">
         <f aca="false">SUM(D7:D20)</f>
-        <v>2962.699</v>
+        <v>2841.0745</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4821,15 +4821,15 @@
       </c>
       <c r="B22" s="4" t="n">
         <f aca="false">B21-SUM(B18:B20)</f>
-        <v>2318.475</v>
+        <v>2211.8505</v>
       </c>
       <c r="C22" s="4" t="n">
         <f aca="false">C21-SUM(C18:C20)</f>
-        <v>2468.6665</v>
+        <v>2282.9335</v>
       </c>
       <c r="D22" s="4" t="n">
         <f aca="false">D21-SUM(D18:D20)</f>
-        <v>2703.699</v>
+        <v>2597.0745</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4855,15 +4855,15 @@
       </c>
       <c r="B24" s="4" t="n">
         <f aca="false">B23-B21</f>
-        <v>122.525</v>
+        <v>244.1495</v>
       </c>
       <c r="C24" s="4" t="n">
         <f aca="false">C23-C21</f>
-        <v>-27.6665000000003</v>
+        <v>173.0665</v>
       </c>
       <c r="D24" s="4" t="n">
         <f aca="false">D23-D21</f>
-        <v>-262.699</v>
+        <v>-141.0745</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4925,15 +4925,15 @@
       </c>
       <c r="B31" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$59*Inputs!$B$6</f>
-        <v>777.327</v>
+        <v>647.7725</v>
       </c>
       <c r="C31" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$59*Inputs!$B$6</f>
-        <v>777.327</v>
+        <v>647.7725</v>
       </c>
       <c r="D31" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$59*Inputs!$B$6</f>
-        <v>777.327</v>
+        <v>647.7725</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="C34" s="4" t="n">
         <f aca="false">Inputs!$B$76*Inputs!$B$63*Inputs!$B$6</f>
-        <v>158.217</v>
+        <v>79.1085</v>
       </c>
       <c r="D34" s="4" t="n">
         <f aca="false">Inputs!$B$62*Inputs!$B$6</f>
@@ -5004,15 +5004,15 @@
       </c>
       <c r="B36" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
-        <v>85.9875</v>
+        <v>68.79</v>
       </c>
       <c r="C36" s="4" t="n">
         <f aca="false">Inputs!$B$76*Inputs!$B$64*Inputs!$B$6</f>
-        <v>34.395</v>
+        <v>17.1975</v>
       </c>
       <c r="D36" s="4" t="n">
         <f aca="false">Inputs!$B$75*Inputs!$B$64*Inputs!$B$6</f>
-        <v>85.9875</v>
+        <v>68.79</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5072,15 +5072,15 @@
       </c>
       <c r="B40" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C40" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="D40" s="4" t="n">
         <f aca="false">Inputs!$B$57*Inputs!$B$74</f>
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5123,15 +5123,15 @@
       </c>
       <c r="B43" s="12" t="n">
         <f aca="false">SUM(B29:B42)</f>
-        <v>2774.673</v>
+        <v>2612.921</v>
       </c>
       <c r="C43" s="12" t="n">
         <f aca="false">SUM(C29:C42)</f>
-        <v>2924.8645</v>
+        <v>2684.004</v>
       </c>
       <c r="D43" s="12" t="n">
         <f aca="false">SUM(D29:D42)</f>
-        <v>3159.897</v>
+        <v>2998.145</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5140,15 +5140,15 @@
       </c>
       <c r="B44" s="4" t="n">
         <f aca="false">B43-SUM(B40:B42)</f>
-        <v>2515.673</v>
+        <v>2368.921</v>
       </c>
       <c r="C44" s="4" t="n">
         <f aca="false">C43-SUM(C40:C42)</f>
-        <v>2665.8645</v>
+        <v>2440.004</v>
       </c>
       <c r="D44" s="4" t="n">
         <f aca="false">D43-SUM(D40:D42)</f>
-        <v>2900.897</v>
+        <v>2754.145</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5174,15 +5174,15 @@
       </c>
       <c r="B46" s="4" t="n">
         <f aca="false">B45-B43</f>
-        <v>-74.6730000000002</v>
+        <v>87.0789999999997</v>
       </c>
       <c r="C46" s="4" t="n">
         <f aca="false">C45-C43</f>
-        <v>-224.8645</v>
+        <v>15.9960000000001</v>
       </c>
       <c r="D46" s="4" t="n">
         <f aca="false">D45-D43</f>
-        <v>-459.897</v>
+        <v>-298.145</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5273,15 +5273,15 @@
       </c>
       <c r="B55" s="4" t="n">
         <f aca="false">B9+B8+B12</f>
-        <v>1028.4105</v>
+        <v>938.9835</v>
       </c>
       <c r="C55" s="4" t="n">
         <f aca="false">B9+B8+B12</f>
-        <v>1028.4105</v>
+        <v>938.9835</v>
       </c>
       <c r="D55" s="4" t="n">
         <f aca="false">B9+B8+B12</f>
-        <v>1028.4105</v>
+        <v>938.9835</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5290,15 +5290,15 @@
       </c>
       <c r="B56" s="4" t="n">
         <f aca="false">B21</f>
-        <v>2577.475</v>
+        <v>2455.8505</v>
       </c>
       <c r="C56" s="4" t="n">
         <f aca="false">B21</f>
-        <v>2577.475</v>
+        <v>2455.8505</v>
       </c>
       <c r="D56" s="4" t="n">
         <f aca="false">B21</f>
-        <v>2577.475</v>
+        <v>2455.8505</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5307,15 +5307,15 @@
       </c>
       <c r="B57" s="4" t="n">
         <f aca="false">MIN(B54,1)*B55</f>
-        <v>1028.4105</v>
+        <v>938.9835</v>
       </c>
       <c r="C57" s="4" t="n">
         <f aca="false">MIN(C54,1)*C55</f>
-        <v>1028.4105</v>
+        <v>938.9835</v>
       </c>
       <c r="D57" s="4" t="n">
         <f aca="false">MIN(D54,1)*D55</f>
-        <v>1028.4105</v>
+        <v>938.9835</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5329,15 +5329,15 @@
       </c>
       <c r="B60" s="4" t="n">
         <f aca="false">B56-B57</f>
-        <v>1549.0645</v>
+        <v>1516.867</v>
       </c>
       <c r="C60" s="4" t="n">
         <f aca="false">C56-C57</f>
-        <v>1549.0645</v>
+        <v>1516.867</v>
       </c>
       <c r="D60" s="4" t="n">
         <f aca="false">D56-D57</f>
-        <v>1549.0645</v>
+        <v>1516.867</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5365,15 +5365,15 @@
       </c>
       <c r="B63" s="5" t="n">
         <f aca="false">(B56-B57)/B53</f>
-        <v>110.647464285714</v>
+        <v>108.347642857143</v>
       </c>
       <c r="C63" s="5" t="n">
         <f aca="false">(C56-C57)/C53</f>
-        <v>81.5297105263158</v>
+        <v>79.8351052631579</v>
       </c>
       <c r="D63" s="5" t="n">
         <f aca="false">(D56-D57)/D53</f>
-        <v>64.5443541666667</v>
+        <v>63.2027916666667</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5382,15 +5382,15 @@
       </c>
       <c r="B64" s="4" t="n">
         <f aca="false">B21+B63</f>
-        <v>2688.12246428571</v>
+        <v>2564.19814285714</v>
       </c>
       <c r="C64" s="4" t="n">
         <f aca="false">B21+C63</f>
-        <v>2659.00471052632</v>
+        <v>2535.68560526316</v>
       </c>
       <c r="D64" s="4" t="n">
         <f aca="false">B21+D63</f>
-        <v>2642.01935416667</v>
+        <v>2519.05329166667</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5399,15 +5399,15 @@
       </c>
       <c r="B65" s="4" t="n">
         <f aca="false">C21+B63</f>
-        <v>2838.31396428571</v>
+        <v>2635.28114285714</v>
       </c>
       <c r="C65" s="4" t="n">
         <f aca="false">C21+C63</f>
-        <v>2809.19621052632</v>
+        <v>2606.76860526316</v>
       </c>
       <c r="D65" s="4" t="n">
         <f aca="false">C21+D63</f>
-        <v>2792.21085416667</v>
+        <v>2590.13629166667</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5421,15 +5421,15 @@
       </c>
       <c r="B67" s="5" t="n">
         <f aca="false">B56/B53</f>
-        <v>184.105357142857</v>
+        <v>175.417892857143</v>
       </c>
       <c r="C67" s="5" t="n">
         <f aca="false">B56/C53</f>
-        <v>135.656578947368</v>
+        <v>129.255289473684</v>
       </c>
       <c r="D67" s="5" t="n">
         <f aca="false">B56/D53</f>
-        <v>107.394791666667</v>
+        <v>102.327104166667</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5438,15 +5438,15 @@
       </c>
       <c r="B68" s="4" t="n">
         <f aca="false">B21+B67</f>
-        <v>2761.58035714286</v>
+        <v>2631.26839285714</v>
       </c>
       <c r="C68" s="4" t="n">
         <f aca="false">B21+C67</f>
-        <v>2713.13157894737</v>
+        <v>2585.10578947368</v>
       </c>
       <c r="D68" s="4" t="n">
         <f aca="false">B21+D67</f>
-        <v>2684.86979166667</v>
+        <v>2558.17760416667</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5455,15 +5455,15 @@
       </c>
       <c r="B69" s="4" t="n">
         <f aca="false">C21+B67</f>
-        <v>2911.77185714286</v>
+        <v>2702.35139285714</v>
       </c>
       <c r="C69" s="4" t="n">
         <f aca="false">C21+C67</f>
-        <v>2863.32307894737</v>
+        <v>2656.18878947368</v>
       </c>
       <c r="D69" s="4" t="n">
         <f aca="false">C21+D67</f>
-        <v>2835.06129166667</v>
+        <v>2629.26060416667</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="D70" s="5" t="n">
         <f aca="false">MAX(D54-1,0)*D55/D53</f>
-        <v>42.8504375</v>
+        <v>39.1243125</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5538,15 +5538,15 @@
       </c>
       <c r="B77" s="4" t="n">
         <f aca="false">B21-B7+B76</f>
-        <v>2277.475</v>
+        <v>2155.8505</v>
       </c>
       <c r="C77" s="4" t="n">
         <f aca="false">B21-B7+C76</f>
-        <v>2577.475</v>
+        <v>2455.8505</v>
       </c>
       <c r="D77" s="4" t="n">
         <f aca="false">B21-B7+D76</f>
-        <v>2877.475</v>
+        <v>2755.8505</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5555,15 +5555,15 @@
       </c>
       <c r="B78" s="4" t="n">
         <f aca="false">C21-B7+B76</f>
-        <v>2427.6665</v>
+        <v>2226.9335</v>
       </c>
       <c r="C78" s="4" t="n">
         <f aca="false">C21-B7+C76</f>
-        <v>2727.6665</v>
+        <v>2526.9335</v>
       </c>
       <c r="D78" s="4" t="n">
         <f aca="false">C21-B7+D76</f>
-        <v>3027.6665</v>
+        <v>2826.9335</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5572,15 +5572,15 @@
       </c>
       <c r="B79" s="4" t="n">
         <f aca="false">D21-B7+B76</f>
-        <v>2662.699</v>
+        <v>2541.0745</v>
       </c>
       <c r="C79" s="4" t="n">
         <f aca="false">D21-B7+C76</f>
-        <v>2962.699</v>
+        <v>2841.0745</v>
       </c>
       <c r="D79" s="4" t="n">
         <f aca="false">D21-B7+D76</f>
-        <v>3262.699</v>
+        <v>3141.0745</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="B80" s="4" t="n">
         <f aca="false">B21-B7+Inputs!$B$55-B8+2*Inputs!$B$69*Inputs!$B$6</f>
-        <v>2833.908</v>
+        <v>2712.2835</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5629,15 +5629,15 @@
       </c>
       <c r="B84" s="4" t="n">
         <f aca="false">(B7+B18+B19+B20)+(B21-(B7+B18+B19+B20))*B83/Inputs!$B$6</f>
-        <v>2445.6275</v>
+        <v>2334.66545</v>
       </c>
       <c r="C84" s="4" t="n">
         <f aca="false">(B7+B18+B19+B20)+(B21-(B7+B18+B19+B20))*C83/Inputs!$B$6</f>
-        <v>2577.475</v>
+        <v>2455.8505</v>
       </c>
       <c r="D84" s="4" t="n">
         <f aca="false">(B7+B18+B19+B20)+(B21-(B7+B18+B19+B20))*D83/Inputs!$B$6</f>
-        <v>2709.3225</v>
+        <v>2577.03555</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5646,15 +5646,15 @@
       </c>
       <c r="B85" s="4" t="n">
         <f aca="false">(C7+C18+C19+C20)+(C21-(C7+C18+C19+C20))*B83/Inputs!$B$6</f>
-        <v>2580.79985</v>
+        <v>2398.64015</v>
       </c>
       <c r="C85" s="4" t="n">
         <f aca="false">(C7+C18+C19+C20)+(C21-(C7+C18+C19+C20))*C83/Inputs!$B$6</f>
-        <v>2727.6665</v>
+        <v>2526.9335</v>
       </c>
       <c r="D85" s="4" t="n">
         <f aca="false">(C7+C18+C19+C20)+(C21-(C7+C18+C19+C20))*D83/Inputs!$B$6</f>
-        <v>2874.53315</v>
+        <v>2655.22685</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5668,7 +5668,7 @@
       </c>
       <c r="B89" s="4" t="n">
         <f aca="false">B56-B55</f>
-        <v>1549.0645</v>
+        <v>1516.867</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5677,7 +5677,7 @@
       </c>
       <c r="B90" s="4" t="n">
         <f aca="false">Inputs!$B$17-B21</f>
-        <v>122.525</v>
+        <v>244.1495</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="B91" s="2" t="n">
         <f aca="false">IF(B90&gt;0,ROUNDUP(B89/B90,0)+1,"not viable at this price")</f>
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5695,16 +5695,16 @@
       </c>
       <c r="B92" s="4" t="n">
         <f aca="false">Inputs!$B$17-C21</f>
-        <v>-27.6665000000003</v>
+        <v>173.0665</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B93" s="2" t="str">
+      <c r="B93" s="2" t="n">
         <f aca="false">IF(B92&gt;0,ROUNDUP(B89/B92,0)+1,"not viable at this price")</f>
-        <v>not viable at this price</v>
+        <v>10</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5754,7 +5754,7 @@
       </c>
       <c r="C100" s="4" t="n">
         <f aca="false">0.5*(B9+B8+B12)</f>
-        <v>514.20525</v>
+        <v>469.49175</v>
       </c>
       <c r="D100" s="2" t="s">
         <v>313</v>
@@ -5783,7 +5783,7 @@
       </c>
       <c r="C102" s="4" t="n">
         <f aca="false">B21-700</f>
-        <v>1877.475</v>
+        <v>1755.8505</v>
       </c>
       <c r="D102" s="2" t="s">
         <v>267</v>

</xml_diff>